<commit_message>
Airbnb-Prüfung: 60-m²-Apartment mit Marktdaten Werlte Q4 2026 (Excel, Präsentation, Businessplan)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Bankunterlagen_Baufeld3.xlsx
+++ b/praesentation/Bankunterlagen_Baufeld3.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="585">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="591">
   <si>
     <t xml:space="preserve">Neue Mitte Werlte, Baufeld 3: Bankunterlagen</t>
   </si>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Darlehen / Beleihungswert</t>
   </si>
   <si>
-    <t xml:space="preserve">Airbnb für 2 Apartments</t>
+    <t xml:space="preserve">Airbnb für 1 Apartment (60 m²)</t>
   </si>
   <si>
     <t xml:space="preserve">Alle Beträge sind Planungsannahmen. KfW-Zinsen und Rahmen sind Stand Ratgeber Oktober 2026 und müssen bei Hausbank und KfW bestätigt werden.</t>
@@ -1524,19 +1524,19 @@
     <t xml:space="preserve">Vereinfachte Rechnung, Hausbank prüft mit eigenen Annahmen.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prüfung: 2 Wohnungen als Airbnb-Apartments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lohnt sich Kurzzeitvermietung gegenüber langfristiger Vermietung? Zwei Apartments, Möblierung im Kredit (Hausbank-Zins + Tilgung).</t>
+    <t xml:space="preserve">Prüfung: 60-m²-Apartment als Airbnb in Werlte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lohnt sich Kurzzeitvermietung gegenüber langfristiger Vermietung? Ein Apartment mit 60 m², Marktdaten Werlte Stand Okt. 2026, Möblierung im Kredit (Hausbank-Zins + Tilgung).</t>
   </si>
   <si>
     <t xml:space="preserve">Eingaben</t>
   </si>
   <si>
-    <t xml:space="preserve">Auslastung Airbnb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annahme; Emsland laut Quelle ca. 37 % (2016/17)</t>
+    <t xml:space="preserve">Preis pro Nacht (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marktschnitt Werlte ca. 87 € (ferienhausmiete.de), 89 % der Angebote unter 100 €; Neubau Zentrum 90 €</t>
   </si>
   <si>
     <t xml:space="preserve">Möblierung je m² (€)</t>
@@ -1557,28 +1557,25 @@
     <t xml:space="preserve">Annahme: Gäste, Schlüssel, Preise kosten Zeit</t>
   </si>
   <si>
-    <t xml:space="preserve">Apartmentgröße (2 Apartments)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">55 m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67 m²</t>
+    <t xml:space="preserve">Apartment 60 m², Szenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Werlte amtlich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emsland-Schnitt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimistisch</t>
   </si>
   <si>
     <t xml:space="preserve">Wohnfläche je Apartment (m²)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gäste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preis pro Nacht (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annahme: kleinere Apartments erzielen mehr Umsatz je m²</t>
+    <t xml:space="preserve">Auslastung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17,4 % Werlte (LSN, Betriebe ab 10 Betten), 36,2 % Emsland, 60 % Annahme Monteure/Business</t>
   </si>
   <si>
     <t xml:space="preserve">Umsatz pro Apartment und Monat</t>
@@ -1602,16 +1599,37 @@
     <t xml:space="preserve">Mehrertrag Airbnb je Apartment pro Monat</t>
   </si>
   <si>
-    <t xml:space="preserve">Mehrertrag für 2 Apartments pro Monat</t>
+    <t xml:space="preserve">Mehrertrag für das Apartment pro Monat</t>
   </si>
   <si>
     <t xml:space="preserve">Ergebnis</t>
   </si>
   <si>
+    <t xml:space="preserve">Break-even Auslastung (Airbnb = langfristige Miete)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fazit</t>
   </si>
   <si>
     <t xml:space="preserve">Die Möblierung erhöht den Kredit, Kurzzeitvermietung braucht dazu Aufwand, Reinigung, Gästekommunikation und bei mehr als 12 Betten Sonderbau-Brandschutz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marktanalyse Werlte (49757), Stand Q4 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auslastung Beherbergung Samtgemeinde Werlte 17,4 % bei 4 Betrieben, 2,7 Tage Aufenthalt, 29.141 Übernachtungen; Emsland gesamt 36,2 % (Emsland Tourismus, Quelle LSN, Betriebe ab 10 Betten).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angebotspreise Werlte im Schnitt ca. 87 € pro Nacht, 89 % der Ferienunterkünfte unter 100 €; Niedersachsen 2025 Rekord mit 46,9 Mio. Übernachtungen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergleich Kleinstadt Diepholz: Airbnb-Auslastung typisch 49 % (Drittanbieter-Schätzung), Spitzenobjekte bis 77 %.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Langfristige Vermietung: Ø 8,79 €/m² Werlte (wohnungsboerse.net, Mai 2026), Annahme Neubau Zentrum 11,18 €/m².</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keine AirDNA-Daten für Werlte verfügbar; Auslastung und Preise sind Näherungen aus Statistik und Portalen.</t>
   </si>
   <si>
     <t xml:space="preserve">Unterlagen für die Bank (Checkliste)</t>
@@ -2633,11 +2651,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="24101086"/>
-        <c:axId val="77528785"/>
+        <c:axId val="43335928"/>
+        <c:axId val="42367973"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24101086"/>
+        <c:axId val="43335928"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2703,7 +2721,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77528785"/>
+        <c:crossAx val="42367973"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2711,7 +2729,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77528785"/>
+        <c:axId val="42367973"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2787,7 +2805,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24101086"/>
+        <c:crossAx val="43335928"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3363,7 +3381,7 @@
       </c>
       <c r="B32" s="15" t="str">
         <f aca="false">'Airbnb Prüfung'!A23</f>
-        <v>Kein Apartment erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
+        <v>Kein Szenario erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
       </c>
       <c r="C32" s="15"/>
     </row>
@@ -4938,7 +4956,7 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -4965,8 +4983,8 @@
       <c r="A4" s="7" t="s">
         <v>499</v>
       </c>
-      <c r="B4" s="20" t="n">
-        <v>0.5</v>
+      <c r="B4" s="19" t="n">
+        <v>90</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>500</v>
@@ -5027,171 +5045,174 @@
         <v>511</v>
       </c>
       <c r="B10" s="18" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>512</v>
       </c>
-      <c r="B11" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>4</v>
+      <c r="B11" s="20" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>513</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>513</v>
-      </c>
-      <c r="B12" s="19" t="n">
-        <v>80</v>
-      </c>
-      <c r="C12" s="19" t="n">
+        <v>499</v>
+      </c>
+      <c r="B12" s="33" t="n">
+        <f aca="false">$B$4</f>
         <v>90</v>
       </c>
-      <c r="D12" s="19" t="n">
-        <v>105</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>514</v>
+      <c r="C12" s="33" t="n">
+        <f aca="false">$B$4</f>
+        <v>90</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <f aca="false">$B$4</f>
+        <v>90</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B13" s="33" t="n">
-        <f aca="false">B12*365*$B$4/12</f>
-        <v>1216.66666666667</v>
+        <f aca="false">B12*365*B11/12</f>
+        <v>476.325</v>
       </c>
       <c r="C13" s="33" t="n">
-        <f aca="false">C12*365*$B$4/12</f>
-        <v>1368.75</v>
+        <f aca="false">C12*365*C11/12</f>
+        <v>990.975</v>
       </c>
       <c r="D13" s="33" t="n">
-        <f aca="false">D12*365*$B$4/12</f>
-        <v>1596.875</v>
+        <f aca="false">D12*365*D11/12</f>
+        <v>1642.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B14" s="33" t="n">
         <f aca="false">B13*(1-$B$6)</f>
-        <v>535.333333333333</v>
+        <v>209.583</v>
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">C13*(1-$B$6)</f>
-        <v>602.25</v>
+        <v>436.029</v>
       </c>
       <c r="D14" s="33" t="n">
         <f aca="false">D13*(1-$B$6)</f>
-        <v>702.625</v>
+        <v>722.7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B15" s="33" t="n">
         <f aca="false">B10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>452.647058823529</v>
+        <v>603.529411764706</v>
       </c>
       <c r="C15" s="33" t="n">
         <f aca="false">C10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>553.235294117647</v>
+        <v>603.529411764706</v>
       </c>
       <c r="D15" s="33" t="n">
         <f aca="false">D10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>673.941176470588</v>
+        <v>603.529411764706</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B16" s="33" t="n">
         <f aca="false">B10*$B$5</f>
-        <v>27000</v>
+        <v>36000</v>
       </c>
       <c r="C16" s="33" t="n">
         <f aca="false">C10*$B$5</f>
-        <v>33000</v>
+        <v>36000</v>
       </c>
       <c r="D16" s="33" t="n">
         <f aca="false">D10*$B$5</f>
-        <v>40200</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B17" s="33" t="n">
         <f aca="false">-B16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-112.5</v>
+        <v>-150</v>
       </c>
       <c r="C17" s="33" t="n">
         <f aca="false">-C16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-137.5</v>
+        <v>-150</v>
       </c>
       <c r="D17" s="33" t="n">
         <f aca="false">-D16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-167.5</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="29" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B18" s="52" t="n">
         <f aca="false">B14-B15+B17</f>
-        <v>-29.8137254901961</v>
+        <v>-543.946411764706</v>
       </c>
       <c r="C18" s="52" t="n">
         <f aca="false">C14-C15+C17</f>
-        <v>-88.4852941176471</v>
+        <v>-317.500411764706</v>
       </c>
       <c r="D18" s="52" t="n">
         <f aca="false">D14-D15+D17</f>
-        <v>-138.816176470588</v>
+        <v>-30.8294117647059</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B19" s="51" t="n">
-        <f aca="false">2*B18</f>
-        <v>-59.6274509803923</v>
+        <f aca="false">B18</f>
+        <v>-543.946411764706</v>
       </c>
       <c r="C19" s="51" t="n">
-        <f aca="false">2*C18</f>
-        <v>-176.970588235294</v>
+        <f aca="false">C18</f>
+        <v>-317.500411764706</v>
       </c>
       <c r="D19" s="51" t="n">
-        <f aca="false">2*D18</f>
-        <v>-277.632352941177</v>
+        <f aca="false">D18</f>
+        <v>-30.8294117647059</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B20" s="29" t="str">
         <f aca="false">IF(B19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
@@ -5206,6 +5227,23 @@
         <v>lohnt sich nicht</v>
       </c>
     </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="B21" s="40" t="n">
+        <f aca="false">(B15-B17)/(B12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <f aca="false">(C15-C17)/(C12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+      <c r="D21" s="40" t="n">
+        <f aca="false">(D15-D17)/(D12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+    </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="43" t="s">
         <v>524</v>
@@ -5213,13 +5251,43 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="43" t="str">
-        <f aca="false">IF(MAX(B19:D19)&gt;=B7,"Mindestens eine Größe erreicht den Mindest-Mehrertrag: Airbnb prüfen.","Kein Apartment erreicht den Mindest-Mehrertrag von "&amp;TEXT(B7,"#,##0")&amp;" € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.")</f>
-        <v>Kein Apartment erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
+        <f aca="false">IF(MAX(B19:D19)&gt;=B7,"Mindestens ein Szenario erreicht den Mindest-Mehrertrag: Airbnb prüfen.","Kein Szenario erreicht den Mindest-Mehrertrag von "&amp;TEXT(B7,"#,##0")&amp;" € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.")</f>
+        <v>Kein Szenario erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
         <v>525</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="43" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -5250,26 +5318,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5277,13 +5345,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C5" s="58" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5291,13 +5359,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="57" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="D6" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5305,13 +5373,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="57" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="D7" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5319,13 +5387,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="57" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="D8" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5333,13 +5401,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="57" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="C9" s="58" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D9" s="59" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5347,13 +5415,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="57" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C10" s="58" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="D10" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5361,13 +5429,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="57" t="s">
+        <v>553</v>
+      </c>
+      <c r="C11" s="58" t="s">
+        <v>554</v>
+      </c>
+      <c r="D11" s="59" t="s">
         <v>547</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>548</v>
-      </c>
-      <c r="D11" s="59" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5375,13 +5443,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="57" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="D12" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5389,13 +5457,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="57" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="C13" s="58" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="D13" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5403,13 +5471,13 @@
         <v>10</v>
       </c>
       <c r="B14" s="57" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C14" s="58" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="D14" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5417,13 +5485,13 @@
         <v>11</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="C15" s="58" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="D15" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5431,13 +5499,13 @@
         <v>12</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C16" s="58" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="D16" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5445,13 +5513,13 @@
         <v>13</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="C17" s="58" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="D17" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5459,13 +5527,13 @@
         <v>14</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="C18" s="58" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="D18" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5473,13 +5541,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="57" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="D19" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5487,13 +5555,13 @@
         <v>16</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="C20" s="58" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="D20" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5501,13 +5569,13 @@
         <v>17</v>
       </c>
       <c r="B21" s="57" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="C21" s="58" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="D21" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5515,13 +5583,13 @@
         <v>18</v>
       </c>
       <c r="B22" s="57" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="C22" s="58" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="D22" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5529,13 +5597,13 @@
         <v>19</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="C23" s="58" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="D23" s="59" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5543,13 +5611,13 @@
         <v>20</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="C24" s="58" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="D24" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5557,13 +5625,13 @@
         <v>21</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C25" s="58" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="D25" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5571,13 +5639,13 @@
         <v>22</v>
       </c>
       <c r="B26" s="57" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="C26" s="58" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="D26" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5585,13 +5653,13 @@
         <v>23</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="C27" s="58" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="D27" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5599,13 +5667,13 @@
         <v>24</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="C28" s="58" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="D28" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5613,13 +5681,13 @@
         <v>25</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="C29" s="58" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="D29" s="59" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gastro: Tagesteil-Umsatzmodell (Frühstück, Mittag, Abend, Bar, Events) mit Abend-Fokus in Excel, Decks und Businessplan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Bankunterlagen_Baufeld3.xlsx
+++ b/praesentation/Bankunterlagen_Baufeld3.xlsx
@@ -18,11 +18,12 @@
     <sheet name="Tilgungsplan" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Ertrag und Cashflow" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Gastro Betrieb" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="Ertragswert" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="Prognose" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="Sensitivität" sheetId="13" state="visible" r:id="rId15"/>
-    <sheet name="Airbnb Prüfung" sheetId="14" state="visible" r:id="rId16"/>
-    <sheet name="Bankunterlagen" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Gastro Tagesteile" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Ertragswert" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Prognose" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="Sensitivität" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="Airbnb Prüfung" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Bankunterlagen" sheetId="16" state="visible" r:id="rId18"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="756" uniqueCount="620">
   <si>
     <t xml:space="preserve">Neue Mitte Werlte, Baufeld 3: Bankunterlagen</t>
   </si>
@@ -147,7 +148,7 @@
     <t xml:space="preserve">Betriebsergebnis Gastro nach Pacht pro Monat</t>
   </si>
   <si>
-    <t xml:space="preserve">bei 65.000 € Umsatz, ohne Lohn des Bauherrn</t>
+    <t xml:space="preserve">bei dem Umsatz aus Blatt Gastro Tagesteile, ohne Lohn des Bauherrn</t>
   </si>
   <si>
     <t xml:space="preserve">Ergebnis pro Monat nach Kapitaldienst</t>
@@ -444,7 +445,7 @@
     <t xml:space="preserve">Gastro-Umsatz pro Monat (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">netto; ca. 4.100 € je Sitzplatz und Jahr bei 190 Plätzen (Österreich Median ca. 12.000 €, vorsichtig)</t>
+    <t xml:space="preserve">netto; Summe aus Frühstück, Mittag, Abend, Bar und Events (Blatt Gastro Tagesteile), Annahmen</t>
   </si>
   <si>
     <t xml:space="preserve">Gastro-Marge vor Pacht</t>
@@ -786,7 +787,7 @@
     <t xml:space="preserve">Gastro-Umsatz je Platz und Jahr (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">vorsichtig, Österreich Median ca. 12.000 €</t>
+    <t xml:space="preserve">Österreich Median ca. 12.000 €</t>
   </si>
   <si>
     <t xml:space="preserve">Pacht in % vom Gastro-Umsatz</t>
@@ -1300,6 +1301,93 @@
   </si>
   <si>
     <t xml:space="preserve">Bei sehr niedrigem Umsatz drücken Fixkosten stärker: die Rechnung ist dort zu günstig.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastro-Umsatz nach Tagesteilen: Frühstück, Mittag, Abend, Bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauptfokus Abend mit Restaurant und Bar. Öffnungstage, Gäste und Bon sind Annahmen (keine Marktdaten für Werlte), Ruhetag Montag.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tagesteil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tage / Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gäste / Tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ø Bon (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz / Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frühstück werktags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di–Fr 08:00–11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brunch am Wochenende</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sa, So 09:00–14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mittagstisch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di–Fr 11:30–14:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abendessen Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di–So 17:30–22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Di–Do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ab 21:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Fr, Sa (bis 01:00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cocktails, Wein, Bier, Musik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feiern, Live-Abende, Séparée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nach Absprache, 4 pro Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastro-Umsatz pro Monat (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">davon Tag (Frühstück, Brunch, Mittag)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">davon Abend (Restaurant, Bar, Feiern)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gäste pro Monat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz je Platz und Jahr (190 Plätze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auslastung der Plätze am Abend (Restaurantgäste je Tag / Plätze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einordnung: Der Abend (Restaurant, Bar, Feiern) trägt den größten Teil des Umsatzes, Frühstück und Mittagstisch füllen das Haus am Tag. Terrasse im Sommer, Catering und Weihnachtsfeiern sind nicht eingerechnet. Branchen-Median Österreich ca. 12.000 € je Platz und Jahr.</t>
   </si>
   <si>
     <t xml:space="preserve">Ertragswert und Beleihung</t>
@@ -2004,7 +2092,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2230,6 +2318,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2651,11 +2743,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="43335928"/>
-        <c:axId val="42367973"/>
+        <c:axId val="85622033"/>
+        <c:axId val="35587217"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43335928"/>
+        <c:axId val="85622033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2721,7 +2813,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42367973"/>
+        <c:crossAx val="35587217"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2729,7 +2821,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42367973"/>
+        <c:axId val="35587217"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2805,7 +2897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43335928"/>
+        <c:crossAx val="85622033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3289,7 +3381,7 @@
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">'Ertrag und Cashflow'!B10</f>
-        <v>14725</v>
+        <v>24068.675</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>37</v>
@@ -3301,7 +3393,7 @@
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>9610.17230350448</v>
+        <v>18953.8473035045</v>
       </c>
       <c r="C25" s="9"/>
     </row>
@@ -3311,7 +3403,7 @@
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">'Ertrag und Cashflow'!B15</f>
-        <v>1.54192628304023</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>40</v>
@@ -3450,7 +3542,7 @@
       <c r="B5" s="7"/>
       <c r="C5" s="10" t="n">
         <f aca="false">Annahmen!$B$49</f>
-        <v>65000</v>
+        <v>95635</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3462,7 +3554,7 @@
       </c>
       <c r="C6" s="33" t="n">
         <f aca="false">-$C$5*B6</f>
-        <v>-18200</v>
+        <v>-26777.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3474,7 +3566,7 @@
       </c>
       <c r="C7" s="33" t="n">
         <f aca="false">-$C$5*B7</f>
-        <v>-19500</v>
+        <v>-28690.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,7 +3578,7 @@
       </c>
       <c r="C8" s="33" t="n">
         <f aca="false">-$C$5*B8</f>
-        <v>-1950</v>
+        <v>-2869.05</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3498,7 +3590,7 @@
       </c>
       <c r="C9" s="33" t="n">
         <f aca="false">-$C$5*B9</f>
-        <v>-1300</v>
+        <v>-1912.7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3510,7 +3602,7 @@
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">-$C$5*B10</f>
-        <v>-975</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3522,7 +3614,7 @@
       </c>
       <c r="C11" s="33" t="n">
         <f aca="false">-$C$5*B11</f>
-        <v>-975</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3534,7 +3626,7 @@
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">-$C$5*B12</f>
-        <v>-975</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3546,7 +3638,7 @@
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">-$C$5*B13</f>
-        <v>-650</v>
+        <v>-956.35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3558,7 +3650,7 @@
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">-$C$5*B14</f>
-        <v>-650</v>
+        <v>-956.35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3571,7 +3663,7 @@
       </c>
       <c r="C15" s="35" t="n">
         <f aca="false">SUM(C6:C14)</f>
-        <v>-45175</v>
+        <v>-66466.325</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3584,7 +3676,7 @@
       </c>
       <c r="C16" s="35" t="n">
         <f aca="false">C5+C15</f>
-        <v>19825</v>
+        <v>29168.675</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>414</v>
@@ -3614,7 +3706,7 @@
       </c>
       <c r="C19" s="46" t="n">
         <f aca="false">C16+C17+C18</f>
-        <v>14725</v>
+        <v>24068.675</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3640,67 +3732,68 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="C24" s="33" t="n">
         <f aca="false">A24*$B$16</f>
-        <v>12200</v>
+        <v>15250</v>
       </c>
       <c r="D24" s="50" t="n">
         <f aca="false">C24-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>7100</v>
+        <v>10150</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="n">
-        <v>50000</v>
+        <v>65000</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">A25*$B$16</f>
-        <v>15250</v>
+        <v>19825</v>
       </c>
       <c r="D25" s="50" t="n">
         <f aca="false">C25-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>10150</v>
+        <v>14725</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="n">
-        <v>65000</v>
+        <v>80000</v>
       </c>
       <c r="C26" s="33" t="n">
         <f aca="false">A26*$B$16</f>
-        <v>19825</v>
+        <v>24400</v>
       </c>
       <c r="D26" s="50" t="n">
         <f aca="false">C26-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>14725</v>
+        <v>19300</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="n">
-        <v>80000</v>
+        <f aca="false">Annahmen!$B$49</f>
+        <v>95635</v>
       </c>
       <c r="C27" s="33" t="n">
         <f aca="false">A27*$B$16</f>
-        <v>24400</v>
+        <v>29168.675</v>
       </c>
       <c r="D27" s="50" t="n">
         <f aca="false">C27-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>19300</v>
+        <v>24068.675</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="n">
-        <v>90000</v>
+        <v>110000</v>
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">A28*$B$16</f>
-        <v>27450</v>
+        <v>33550</v>
       </c>
       <c r="D28" s="50" t="n">
         <f aca="false">C28-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>22350</v>
+        <v>28450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,13 +3818,14 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3749,466 +3843,269 @@
         <v>424</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>203</v>
+        <v>425</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>199</v>
+        <v>427</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>204</v>
+        <v>428</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>233</v>
+        <v>429</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>426</v>
-      </c>
-      <c r="B5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!G20</f>
-        <v>87847.0588235294</v>
-      </c>
-      <c r="C5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!G25</f>
-        <v>19200</v>
-      </c>
-      <c r="D5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!G22</f>
-        <v>61200</v>
-      </c>
-      <c r="E5" s="35" t="n">
-        <f aca="false">SUM(B5:D5)</f>
-        <v>168247.058823529</v>
+      <c r="A5" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C5" s="57" t="n">
+        <v>17</v>
+      </c>
+      <c r="D5" s="57" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" s="33" t="n">
+        <f aca="false">C5*D5*E5</f>
+        <v>4675</v>
+      </c>
+      <c r="G5" s="40" t="n">
+        <f aca="false">F5/$F$14</f>
+        <v>0.0488837768599362</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>427</v>
-      </c>
-      <c r="B6" s="33" t="n">
-        <f aca="false">-(Annahmen!$B$24+Annahmen!$B$26)*Annahmen!$B$69</f>
-        <v>-2880</v>
-      </c>
-      <c r="C6" s="33" t="n">
-        <f aca="false">-C5*Annahmen!$B$72</f>
-        <v>-576</v>
-      </c>
-      <c r="D6" s="33" t="n">
-        <f aca="false">-D5*Annahmen!$B$72</f>
-        <v>-1836</v>
+        <v>432</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C6" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="D6" s="57" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <f aca="false">C6*D6*E6</f>
+        <v>7560</v>
+      </c>
+      <c r="G6" s="40" t="n">
+        <f aca="false">F6/$F$14</f>
+        <v>0.0790505568045172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="B7" s="33" t="n">
-        <f aca="false">-(Annahmen!$B$23+Annahmen!$B$25)*Annahmen!$B$70</f>
-        <v>-7860</v>
-      </c>
-      <c r="C7" s="33" t="n">
-        <f aca="false">-(Annahmen!$B$29+Annahmen!$B$31)*Annahmen!$B$73</f>
-        <v>-1320</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <f aca="false">-Annahmen!$B$21*Annahmen!$B$73</f>
-        <v>-4080</v>
+        <v>434</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="C7" s="57" t="n">
+        <v>17</v>
+      </c>
+      <c r="D7" s="57" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <f aca="false">C7*D7*E7</f>
+        <v>11900</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <f aca="false">F7/$F$14</f>
+        <v>0.12443143200711</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>429</v>
-      </c>
-      <c r="B8" s="33" t="n">
-        <f aca="false">-B5*Annahmen!$B$71</f>
-        <v>-1756.94117647059</v>
-      </c>
-      <c r="C8" s="33" t="n">
-        <f aca="false">-C5*Annahmen!$B$75</f>
-        <v>-384</v>
-      </c>
-      <c r="D8" s="33" t="n">
-        <f aca="false">-D5*Annahmen!$B$74</f>
-        <v>-2448</v>
+        <v>436</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="C8" s="57" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" s="57" t="n">
+        <v>55</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" s="33" t="n">
+        <f aca="false">C8*D8*E8</f>
+        <v>45760</v>
+      </c>
+      <c r="G8" s="40" t="n">
+        <f aca="false">F8/$F$14</f>
+        <v>0.478485909970199</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>430</v>
-      </c>
-      <c r="B9" s="35" t="n">
-        <f aca="false">SUM(B6:B8)</f>
-        <v>-12496.9411764706</v>
-      </c>
-      <c r="C9" s="35" t="n">
-        <f aca="false">SUM(C6:C8)</f>
-        <v>-2280</v>
-      </c>
-      <c r="D9" s="35" t="n">
-        <f aca="false">SUM(D6:D8)</f>
-        <v>-8364</v>
-      </c>
-      <c r="E9" s="35" t="n">
-        <f aca="false">SUM(B9:D9)</f>
-        <v>-23140.9411764706</v>
+      <c r="A9" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C9" s="57" t="n">
+        <v>13</v>
+      </c>
+      <c r="D9" s="57" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <f aca="false">C9*D9*E9</f>
+        <v>4680</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <f aca="false">F9/$F$14</f>
+        <v>0.0489360589742249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>431</v>
-      </c>
-      <c r="B10" s="35" t="n">
-        <f aca="false">B5+B9</f>
-        <v>75350.1176470588</v>
-      </c>
-      <c r="C10" s="35" t="n">
-        <f aca="false">C5+C9</f>
-        <v>16920</v>
-      </c>
-      <c r="D10" s="35" t="n">
-        <f aca="false">D5+D9</f>
-        <v>52836</v>
-      </c>
-      <c r="E10" s="35" t="n">
-        <f aca="false">SUM(B10:D10)</f>
-        <v>145106.117647059</v>
+      <c r="A10" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="C10" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="57" t="n">
+        <v>70</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="F10" s="33" t="n">
+        <f aca="false">C10*D10*E10</f>
+        <v>13860</v>
+      </c>
+      <c r="G10" s="40" t="n">
+        <f aca="false">F10/$F$14</f>
+        <v>0.144926020808281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>432</v>
-      </c>
-      <c r="B11" s="40" t="n">
-        <f aca="false">(Annahmen!$B$23+Annahmen!$B$25)/((Annahmen!$B$23+Annahmen!$B$25)+Annahmen!$B$29+Annahmen!$B$31+Annahmen!$B$21)</f>
-        <v>0.492481203007519</v>
-      </c>
-      <c r="C11" s="40" t="n">
-        <f aca="false">(Annahmen!$B$29+Annahmen!$B$31)/((Annahmen!$B$23+Annahmen!$B$25)+Annahmen!$B$29+Annahmen!$B$31+Annahmen!$B$21)</f>
-        <v>0.12406015037594</v>
-      </c>
-      <c r="D11" s="40" t="n">
-        <f aca="false">1-B11-C11</f>
-        <v>0.383458646616541</v>
-      </c>
-      <c r="E11" s="40" t="n">
-        <f aca="false">SUM(B11:D11)</f>
+        <v>442</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="C11" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="57" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" s="33" t="n">
+        <f aca="false">C11*D11*E11</f>
+        <v>7200</v>
+      </c>
+      <c r="G11" s="40" t="n">
+        <f aca="false">F11/$F$14</f>
+        <v>0.0752862445757307</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="29" t="s">
+        <v>444</v>
+      </c>
+      <c r="F14" s="46" t="n">
+        <f aca="false">SUM(F5:F11)</f>
+        <v>95635</v>
+      </c>
+      <c r="G14" s="42" t="n">
+        <f aca="false">SUM(G5:G11)</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="B12" s="33" t="n">
-        <f aca="false">$E$12*B11</f>
-        <v>108739.84962406</v>
-      </c>
-      <c r="C12" s="33" t="n">
-        <f aca="false">$E$12*C11</f>
-        <v>27392.4812030075</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <f aca="false">$E$12*D11</f>
-        <v>84667.6691729323</v>
-      </c>
-      <c r="E12" s="35" t="n">
-        <f aca="false">Annahmen!$B$5*Annahmen!$B$6</f>
-        <v>220800</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="B13" s="12" t="n">
-        <f aca="false">Annahmen!$B$64</f>
-        <v>0.04</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <f aca="false">Annahmen!$B$65</f>
-        <v>0.06</v>
-      </c>
-      <c r="D13" s="12" t="n">
-        <f aca="false">Annahmen!$B$66</f>
-        <v>0.065</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="B14" s="33" t="n">
-        <f aca="false">-B12*B13</f>
-        <v>-4349.59398496241</v>
-      </c>
-      <c r="C14" s="33" t="n">
-        <f aca="false">-C12*C13</f>
-        <v>-1643.54887218045</v>
-      </c>
-      <c r="D14" s="33" t="n">
-        <f aca="false">-D12*D13</f>
-        <v>-5503.3984962406</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>436</v>
-      </c>
-      <c r="B15" s="33" t="n">
-        <f aca="false">B10+B14</f>
-        <v>71000.5236620964</v>
-      </c>
-      <c r="C15" s="33" t="n">
-        <f aca="false">C10+C14</f>
-        <v>15276.4511278196</v>
-      </c>
-      <c r="D15" s="33" t="n">
-        <f aca="false">D10+D14</f>
-        <v>47332.6015037594</v>
-      </c>
-      <c r="E15" s="33" t="n">
-        <f aca="false">SUM(B15:D15)</f>
-        <v>133609.576293675</v>
+        <v>445</v>
+      </c>
+      <c r="F15" s="33" t="n">
+        <f aca="false">SUM(F5:F7)</f>
+        <v>24135</v>
+      </c>
+      <c r="G15" s="40" t="n">
+        <f aca="false">F15/F14</f>
+        <v>0.252365765671564</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>437</v>
-      </c>
-      <c r="B16" s="8" t="n">
-        <f aca="false">Annahmen!$B$67</f>
-        <v>80</v>
-      </c>
-      <c r="C16" s="8" t="n">
-        <f aca="false">Annahmen!$B$68</f>
-        <v>60</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <f aca="false">Annahmen!$B$68</f>
-        <v>60</v>
+      <c r="A16" s="29" t="s">
+        <v>446</v>
+      </c>
+      <c r="F16" s="35" t="n">
+        <f aca="false">SUM(F8:F11)</f>
+        <v>71500</v>
+      </c>
+      <c r="G16" s="42" t="n">
+        <f aca="false">F16/F14</f>
+        <v>0.747634234328436</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="B17" s="39" t="n">
-        <f aca="false">((1+B13)^B16-1)/(B13*(1+B13)^B16)</f>
-        <v>23.915391846835</v>
-      </c>
-      <c r="C17" s="39" t="n">
-        <f aca="false">((1+C13)^C16-1)/(C13*(1+C13)^C16)</f>
-        <v>16.161427705238</v>
-      </c>
-      <c r="D17" s="39" t="n">
-        <f aca="false">((1+D13)^D16-1)/(D13*(1+D13)^D16)</f>
-        <v>15.0329657448345</v>
-      </c>
-      <c r="E17" s="39" t="n">
-        <f aca="false">E18/E15</f>
-        <v>19.882137612542</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>439</v>
+        <v>447</v>
+      </c>
+      <c r="F17" s="28" t="n">
+        <f aca="false">SUMPRODUCT(C5:C11,D5:D11)</f>
+        <v>4295</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>440</v>
-      </c>
-      <c r="B18" s="35" t="n">
-        <f aca="false">B15*B17</f>
-        <v>1698005.34470951</v>
-      </c>
-      <c r="C18" s="35" t="n">
-        <f aca="false">C15*C17</f>
-        <v>246889.260494858</v>
-      </c>
-      <c r="D18" s="35" t="n">
-        <f aca="false">D15*D17</f>
-        <v>711549.377019915</v>
-      </c>
-      <c r="E18" s="35" t="n">
-        <f aca="false">SUM(B18:D18)</f>
-        <v>2656443.98222429</v>
-      </c>
+      <c r="A18" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="F18" s="33" t="n">
+        <f aca="false">F14*12/(Annahmen!$B$36+Annahmen!$B$37)</f>
+        <v>6040.1052631579</v>
+      </c>
+      <c r="G18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="s">
-        <v>441</v>
-      </c>
-      <c r="B19" s="46" t="n">
-        <f aca="false">B18+B12</f>
-        <v>1806745.19433357</v>
-      </c>
-      <c r="C19" s="46" t="n">
-        <f aca="false">C18+C12</f>
-        <v>274281.741697865</v>
-      </c>
-      <c r="D19" s="46" t="n">
-        <f aca="false">D18+D12</f>
-        <v>796217.046192847</v>
-      </c>
-      <c r="E19" s="46" t="n">
-        <f aca="false">SUM(B19:D19)</f>
-        <v>2877243.98222429</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>442</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>443</v>
-      </c>
-      <c r="B23" s="33" t="n">
-        <f aca="false">E12+'Kosten und Finanzierung'!B12+'Kosten und Finanzierung'!B13+'Kosten und Finanzierung'!B14</f>
-        <v>4325625.525</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="33" t="n">
-        <f aca="false">E19</f>
-        <v>2877243.98222429</v>
-      </c>
-      <c r="F24" s="9"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="B25" s="33" t="n">
-        <f aca="false">MIN(B23,B24)</f>
-        <v>2877243.98222429</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
-        <v>447</v>
-      </c>
-      <c r="B26" s="46" t="n">
-        <f aca="false">B25*(1-Annahmen!$B$76)</f>
-        <v>2589519.58400186</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="B27" s="33" t="n">
-        <f aca="false">'Kosten und Finanzierung'!B18</f>
-        <v>4845505.70598245</v>
-      </c>
-      <c r="F27" s="9"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="A19" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="B28" s="33" t="n">
-        <f aca="false">'Kosten und Finanzierung'!B29</f>
-        <v>4845505.70598245</v>
-      </c>
-      <c r="F28" s="9"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="29" t="s">
+      <c r="F19" s="40" t="n">
+        <f aca="false">D8/(Annahmen!$B$36+Annahmen!$B$37)</f>
+        <v>0.289473684210526</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="s">
         <v>450</v>
-      </c>
-      <c r="B29" s="44" t="n">
-        <f aca="false">B28/B26</f>
-        <v>1.87119871033923</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="s">
-        <v>452</v>
-      </c>
-      <c r="B30" s="40" t="n">
-        <f aca="false">('Kosten und Finanzierung'!B24+'Kosten und Finanzierung'!B25+'Kosten und Finanzierung'!B26)/B26</f>
-        <v>0.906538809168673</v>
-      </c>
-      <c r="F30" s="9"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="s">
-        <v>453</v>
-      </c>
-      <c r="B31" s="52" t="n">
-        <f aca="false">E19-B27</f>
-        <v>-1968261.72375817</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="s">
-        <v>455</v>
-      </c>
-      <c r="B32" s="33" t="n">
-        <f aca="false">MAX(0,B28-0.8*B26)</f>
-        <v>2773890.03878097</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>457</v>
-      </c>
-      <c r="B33" s="31" t="n">
-        <f aca="false">E19/E5</f>
-        <v>17.1013032997038</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="s">
-        <v>459</v>
-      </c>
-      <c r="B34" s="31" t="n">
-        <f aca="false">B27/E5</f>
-        <v>28.7999430115732</v>
-      </c>
-      <c r="F34" s="9"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="16" t="s">
-        <v>460</v>
       </c>
     </row>
   </sheetData>
@@ -4228,511 +4125,490 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>344</v>
+        <v>453</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>463</v>
+        <v>203</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>465</v>
+        <v>199</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>466</v>
+        <v>204</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>467</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>471</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>472</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>473</v>
+      <c r="A5" s="29" t="s">
+        <v>455</v>
       </c>
       <c r="B5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(1-1)</f>
+        <f aca="false">'Flächen und Mieten'!G20</f>
         <v>87847.0588235294</v>
       </c>
       <c r="C5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(2-1)</f>
-        <v>89164.7647058823</v>
+        <f aca="false">'Flächen und Mieten'!G25</f>
+        <v>19200</v>
       </c>
       <c r="D5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(3-1)</f>
-        <v>90502.2361764706</v>
-      </c>
-      <c r="E5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(4-1)</f>
-        <v>91859.7697191176</v>
-      </c>
-      <c r="F5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(5-1)</f>
-        <v>93237.6662649044</v>
-      </c>
-      <c r="G5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(6-1)</f>
-        <v>94636.2312588779</v>
-      </c>
-      <c r="H5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(7-1)</f>
-        <v>96055.7747277611</v>
-      </c>
-      <c r="I5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(8-1)</f>
-        <v>97496.6113486775</v>
-      </c>
-      <c r="J5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(9-1)</f>
-        <v>98959.0605189077</v>
-      </c>
-      <c r="K5" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(10-1)</f>
-        <v>100443.446426691</v>
+        <f aca="false">'Flächen und Mieten'!G22</f>
+        <v>61200</v>
+      </c>
+      <c r="E5" s="35" t="n">
+        <f aca="false">SUM(B5:D5)</f>
+        <v>168247.058823529</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>474</v>
+        <v>456</v>
       </c>
       <c r="B6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(1-1)</f>
-        <v>19200</v>
+        <f aca="false">-(Annahmen!$B$24+Annahmen!$B$26)*Annahmen!$B$69</f>
+        <v>-2880</v>
       </c>
       <c r="C6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(2-1)</f>
-        <v>19584</v>
+        <f aca="false">-C5*Annahmen!$B$72</f>
+        <v>-576</v>
       </c>
       <c r="D6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(3-1)</f>
-        <v>19975.68</v>
-      </c>
-      <c r="E6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(4-1)</f>
-        <v>20375.1936</v>
-      </c>
-      <c r="F6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(5-1)</f>
-        <v>20782.697472</v>
-      </c>
-      <c r="G6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(6-1)</f>
-        <v>21198.35142144</v>
-      </c>
-      <c r="H6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(7-1)</f>
-        <v>21622.3184498688</v>
-      </c>
-      <c r="I6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(8-1)</f>
-        <v>22054.7648188662</v>
-      </c>
-      <c r="J6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(9-1)</f>
-        <v>22495.8601152435</v>
-      </c>
-      <c r="K6" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(10-1)</f>
-        <v>22945.7773175484</v>
+        <f aca="false">-D5*Annahmen!$B$72</f>
+        <v>-1836</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>380</v>
+        <v>457</v>
       </c>
       <c r="B7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(1-1)</f>
-        <v>61200</v>
+        <f aca="false">-(Annahmen!$B$23+Annahmen!$B$25)*Annahmen!$B$70</f>
+        <v>-7860</v>
       </c>
       <c r="C7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(2-1)</f>
-        <v>62118</v>
+        <f aca="false">-(Annahmen!$B$29+Annahmen!$B$31)*Annahmen!$B$73</f>
+        <v>-1320</v>
       </c>
       <c r="D7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(3-1)</f>
-        <v>63049.77</v>
-      </c>
-      <c r="E7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(4-1)</f>
-        <v>63995.51655</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(5-1)</f>
-        <v>64955.44929825</v>
-      </c>
-      <c r="G7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(6-1)</f>
-        <v>65929.7810377237</v>
-      </c>
-      <c r="H7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(7-1)</f>
-        <v>66918.7277532896</v>
-      </c>
-      <c r="I7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(8-1)</f>
-        <v>67922.5086695889</v>
-      </c>
-      <c r="J7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(9-1)</f>
-        <v>68941.3462996327</v>
-      </c>
-      <c r="K7" s="33" t="n">
-        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(10-1)</f>
-        <v>69975.4664941272</v>
+        <f aca="false">-Annahmen!$B$21*Annahmen!$B$73</f>
+        <v>-4080</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>475</v>
-      </c>
-      <c r="B8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(B5+B6+B7)</f>
-        <v>-16824.7058823529</v>
-      </c>
-      <c r="C8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(C5+C6+C7)</f>
-        <v>-17086.6764705882</v>
-      </c>
-      <c r="D8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(D5+D6+D7)</f>
-        <v>-17352.7686176471</v>
-      </c>
-      <c r="E8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(E5+E6+E7)</f>
-        <v>-17623.0479869118</v>
-      </c>
-      <c r="F8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(F5+F6+F7)</f>
-        <v>-17897.5813035154</v>
-      </c>
-      <c r="G8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(G5+G6+G7)</f>
-        <v>-18176.4363718042</v>
-      </c>
-      <c r="H8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(H5+H6+H7)</f>
-        <v>-18459.6820930919</v>
-      </c>
-      <c r="I8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(I5+I6+I7)</f>
-        <v>-18747.3884837133</v>
-      </c>
-      <c r="J8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(J5+J6+J7)</f>
-        <v>-19039.6266933784</v>
-      </c>
-      <c r="K8" s="50" t="n">
-        <f aca="false">-Annahmen!$B$48*(K5+K6+K7)</f>
-        <v>-19336.4690238367</v>
+        <v>458</v>
+      </c>
+      <c r="B8" s="33" t="n">
+        <f aca="false">-B5*Annahmen!$B$71</f>
+        <v>-1756.94117647059</v>
+      </c>
+      <c r="C8" s="33" t="n">
+        <f aca="false">-C5*Annahmen!$B$75</f>
+        <v>-384</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <f aca="false">-D5*Annahmen!$B$74</f>
+        <v>-2448</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>385</v>
-      </c>
-      <c r="B9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(1-1))-B7-Annahmen!$B$51*12</f>
-        <v>176700</v>
-      </c>
-      <c r="C9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(2-1))-C7-Annahmen!$B$51*12</f>
-        <v>179350.5</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(3-1))-D7-Annahmen!$B$51*12</f>
-        <v>182040.7575</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(4-1))-E7-Annahmen!$B$51*12</f>
-        <v>184771.3688625</v>
-      </c>
-      <c r="F9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(5-1))-F7-Annahmen!$B$51*12</f>
-        <v>187542.939395437</v>
-      </c>
-      <c r="G9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(6-1))-G7-Annahmen!$B$51*12</f>
-        <v>190356.083486369</v>
-      </c>
-      <c r="H9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(7-1))-H7-Annahmen!$B$51*12</f>
-        <v>193211.424738664</v>
-      </c>
-      <c r="I9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(8-1))-I7-Annahmen!$B$51*12</f>
-        <v>196109.596109744</v>
-      </c>
-      <c r="J9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(9-1))-J7-Annahmen!$B$51*12</f>
-        <v>199051.240051391</v>
-      </c>
-      <c r="K9" s="33" t="n">
-        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(10-1))-K7-Annahmen!$B$51*12</f>
-        <v>202037.008652161</v>
+      <c r="A9" s="29" t="s">
+        <v>459</v>
+      </c>
+      <c r="B9" s="35" t="n">
+        <f aca="false">SUM(B6:B8)</f>
+        <v>-12496.9411764706</v>
+      </c>
+      <c r="C9" s="35" t="n">
+        <f aca="false">SUM(C6:C8)</f>
+        <v>-2280</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <f aca="false">SUM(D6:D8)</f>
+        <v>-8364</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <f aca="false">SUM(B9:D9)</f>
+        <v>-23140.9411764706</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="29" t="s">
-        <v>387</v>
+        <v>460</v>
       </c>
       <c r="B10" s="35" t="n">
-        <f aca="false">SUM(B5:B9)</f>
-        <v>328122.352941176</v>
+        <f aca="false">B5+B9</f>
+        <v>75350.1176470588</v>
       </c>
       <c r="C10" s="35" t="n">
-        <f aca="false">SUM(C5:C9)</f>
-        <v>333130.588235294</v>
+        <f aca="false">C5+C9</f>
+        <v>16920</v>
       </c>
       <c r="D10" s="35" t="n">
-        <f aca="false">SUM(D5:D9)</f>
-        <v>338215.675058823</v>
+        <f aca="false">D5+D9</f>
+        <v>52836</v>
       </c>
       <c r="E10" s="35" t="n">
-        <f aca="false">SUM(E5:E9)</f>
-        <v>343378.800744706</v>
-      </c>
-      <c r="F10" s="35" t="n">
-        <f aca="false">SUM(F5:F9)</f>
-        <v>348621.171127076</v>
-      </c>
-      <c r="G10" s="35" t="n">
-        <f aca="false">SUM(G5:G9)</f>
-        <v>353944.010832606</v>
-      </c>
-      <c r="H10" s="35" t="n">
-        <f aca="false">SUM(H5:H9)</f>
-        <v>359348.563576492</v>
-      </c>
-      <c r="I10" s="35" t="n">
-        <f aca="false">SUM(I5:I9)</f>
-        <v>364836.092463164</v>
-      </c>
-      <c r="J10" s="35" t="n">
-        <f aca="false">SUM(J5:J9)</f>
-        <v>370407.880291796</v>
-      </c>
-      <c r="K10" s="35" t="n">
-        <f aca="false">SUM(K5:K9)</f>
-        <v>376065.229866692</v>
+        <f aca="false">SUM(B10:D10)</f>
+        <v>145106.117647059</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="B11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D5</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="C11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D6</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="D11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D7</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="E11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D8</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="F11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D9</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="G11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D10</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="H11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D11</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="I11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D12</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="J11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D13</f>
-        <v>-212800.285299123</v>
-      </c>
-      <c r="K11" s="50" t="n">
-        <f aca="false">-'Tilgung Jahre'!D14</f>
-        <v>-212800.285299123</v>
+        <v>461</v>
+      </c>
+      <c r="B11" s="40" t="n">
+        <f aca="false">(Annahmen!$B$23+Annahmen!$B$25)/((Annahmen!$B$23+Annahmen!$B$25)+Annahmen!$B$29+Annahmen!$B$31+Annahmen!$B$21)</f>
+        <v>0.492481203007519</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <f aca="false">(Annahmen!$B$29+Annahmen!$B$31)/((Annahmen!$B$23+Annahmen!$B$25)+Annahmen!$B$29+Annahmen!$B$31+Annahmen!$B$21)</f>
+        <v>0.12406015037594</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <f aca="false">1-B11-C11</f>
+        <v>0.383458646616541</v>
+      </c>
+      <c r="E11" s="40" t="n">
+        <f aca="false">SUM(B11:D11)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
-        <v>477</v>
-      </c>
-      <c r="B12" s="52" t="n">
-        <f aca="false">B10+B11</f>
-        <v>115322.067642054</v>
-      </c>
-      <c r="C12" s="52" t="n">
-        <f aca="false">C10+C11</f>
-        <v>120330.302936171</v>
-      </c>
-      <c r="D12" s="52" t="n">
-        <f aca="false">D10+D11</f>
-        <v>125415.389759701</v>
-      </c>
-      <c r="E12" s="52" t="n">
-        <f aca="false">E10+E11</f>
-        <v>130578.515445583</v>
-      </c>
-      <c r="F12" s="52" t="n">
-        <f aca="false">F10+F11</f>
-        <v>135820.885827954</v>
-      </c>
-      <c r="G12" s="52" t="n">
-        <f aca="false">G10+G11</f>
-        <v>141143.725533484</v>
-      </c>
-      <c r="H12" s="52" t="n">
-        <f aca="false">H10+H11</f>
-        <v>146548.278277369</v>
-      </c>
-      <c r="I12" s="52" t="n">
-        <f aca="false">I10+I11</f>
-        <v>152035.807164041</v>
-      </c>
-      <c r="J12" s="52" t="n">
-        <f aca="false">J10+J11</f>
-        <v>157607.594992673</v>
-      </c>
-      <c r="K12" s="52" t="n">
-        <f aca="false">K10+K11</f>
-        <v>163264.944567569</v>
+      <c r="A12" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="B12" s="33" t="n">
+        <f aca="false">$E$12*B11</f>
+        <v>108739.84962406</v>
+      </c>
+      <c r="C12" s="33" t="n">
+        <f aca="false">$E$12*C11</f>
+        <v>27392.4812030075</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <f aca="false">$E$12*D11</f>
+        <v>84667.6691729323</v>
+      </c>
+      <c r="E12" s="35" t="n">
+        <f aca="false">Annahmen!$B$5*Annahmen!$B$6</f>
+        <v>220800</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>478</v>
-      </c>
-      <c r="B13" s="54" t="n">
-        <f aca="false">B10/-B11</f>
-        <v>1.54192628304023</v>
-      </c>
-      <c r="C13" s="54" t="n">
-        <f aca="false">C10/-C11</f>
-        <v>1.56546119177909</v>
-      </c>
-      <c r="D13" s="54" t="n">
-        <f aca="false">D10/-D11</f>
-        <v>1.58935724443889</v>
-      </c>
-      <c r="E13" s="54" t="n">
-        <f aca="false">E10/-E11</f>
-        <v>1.61362002058426</v>
-      </c>
-      <c r="F13" s="54" t="n">
-        <f aca="false">F10/-F11</f>
-        <v>1.63825518672138</v>
-      </c>
-      <c r="G13" s="54" t="n">
-        <f aca="false">G10/-G11</f>
-        <v>1.66326849766712</v>
-      </c>
-      <c r="H13" s="54" t="n">
-        <f aca="false">H10/-H11</f>
-        <v>1.68866579793995</v>
-      </c>
-      <c r="I13" s="54" t="n">
-        <f aca="false">I10/-I11</f>
-        <v>1.71445302317303</v>
-      </c>
-      <c r="J13" s="54" t="n">
-        <f aca="false">J10/-J11</f>
-        <v>1.74063620154988</v>
-      </c>
-      <c r="K13" s="54" t="n">
-        <f aca="false">K10/-K11</f>
-        <v>1.76722145526297</v>
+      <c r="A13" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <f aca="false">Annahmen!$B$64</f>
+        <v>0.04</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <f aca="false">Annahmen!$B$65</f>
+        <v>0.06</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <f aca="false">Annahmen!$B$66</f>
+        <v>0.065</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>348</v>
+        <v>464</v>
       </c>
       <c r="B14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E5</f>
-        <v>4796289.99144002</v>
+        <f aca="false">-B12*B13</f>
+        <v>-4349.59398496241</v>
       </c>
       <c r="C14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E6</f>
-        <v>4745376.85834322</v>
+        <f aca="false">-C12*C13</f>
+        <v>-1643.54887218045</v>
       </c>
       <c r="D14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E7</f>
-        <v>4692705.54860192</v>
-      </c>
-      <c r="E14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E8</f>
-        <v>4638213.05983898</v>
-      </c>
-      <c r="F14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E9</f>
-        <v>4581834.06036832</v>
-      </c>
-      <c r="G14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E10</f>
-        <v>4523500.80088865</v>
-      </c>
-      <c r="H14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E11</f>
-        <v>4463143.02276395</v>
-      </c>
-      <c r="I14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E12</f>
-        <v>4400687.86275702</v>
-      </c>
-      <c r="J14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E13</f>
-        <v>4336059.75407694</v>
-      </c>
-      <c r="K14" s="33" t="n">
-        <f aca="false">'Tilgung Jahre'!E14</f>
-        <v>4269180.3235956</v>
+        <f aca="false">-D12*D13</f>
+        <v>-5503.3984962406</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="B15" s="33" t="n">
+        <f aca="false">B10+B14</f>
+        <v>71000.5236620964</v>
+      </c>
+      <c r="C15" s="33" t="n">
+        <f aca="false">C10+C14</f>
+        <v>15276.4511278196</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <f aca="false">D10+D14</f>
+        <v>47332.6015037594</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <f aca="false">SUM(B15:D15)</f>
+        <v>133609.576293675</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <f aca="false">Annahmen!$B$67</f>
+        <v>80</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <f aca="false">Annahmen!$B$68</f>
+        <v>60</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <f aca="false">Annahmen!$B$68</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="B17" s="39" t="n">
+        <f aca="false">((1+B13)^B16-1)/(B13*(1+B13)^B16)</f>
+        <v>23.915391846835</v>
+      </c>
+      <c r="C17" s="39" t="n">
+        <f aca="false">((1+C13)^C16-1)/(C13*(1+C13)^C16)</f>
+        <v>16.161427705238</v>
+      </c>
+      <c r="D17" s="39" t="n">
+        <f aca="false">((1+D13)^D16-1)/(D13*(1+D13)^D16)</f>
+        <v>15.0329657448345</v>
+      </c>
+      <c r="E17" s="39" t="n">
+        <f aca="false">E18/E15</f>
+        <v>19.882137612542</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="29" t="s">
+        <v>469</v>
+      </c>
+      <c r="B18" s="35" t="n">
+        <f aca="false">B15*B17</f>
+        <v>1698005.34470951</v>
+      </c>
+      <c r="C18" s="35" t="n">
+        <f aca="false">C15*C17</f>
+        <v>246889.260494858</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <f aca="false">D15*D17</f>
+        <v>711549.377019915</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <f aca="false">SUM(B18:D18)</f>
+        <v>2656443.98222429</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="29" t="s">
+        <v>470</v>
+      </c>
+      <c r="B19" s="46" t="n">
+        <f aca="false">B18+B12</f>
+        <v>1806745.19433357</v>
+      </c>
+      <c r="C19" s="46" t="n">
+        <f aca="false">C18+C12</f>
+        <v>274281.741697865</v>
+      </c>
+      <c r="D19" s="46" t="n">
+        <f aca="false">D18+D12</f>
+        <v>796217.046192847</v>
+      </c>
+      <c r="E19" s="46" t="n">
+        <f aca="false">SUM(B19:D19)</f>
+        <v>2877243.98222429</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="B23" s="33" t="n">
+        <f aca="false">E12+'Kosten und Finanzierung'!B12+'Kosten und Finanzierung'!B13+'Kosten und Finanzierung'!B14</f>
+        <v>4325625.525</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="33" t="n">
+        <f aca="false">E19</f>
+        <v>2877243.98222429</v>
+      </c>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="B25" s="33" t="n">
+        <f aca="false">MIN(B23,B24)</f>
+        <v>2877243.98222429</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="29" t="s">
+        <v>476</v>
+      </c>
+      <c r="B26" s="46" t="n">
+        <f aca="false">B25*(1-Annahmen!$B$76)</f>
+        <v>2589519.58400186</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B27" s="33" t="n">
+        <f aca="false">'Kosten und Finanzierung'!B18</f>
+        <v>4845505.70598245</v>
+      </c>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="B28" s="33" t="n">
+        <f aca="false">'Kosten und Finanzierung'!B29</f>
+        <v>4845505.70598245</v>
+      </c>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="29" t="s">
         <v>479</v>
+      </c>
+      <c r="B29" s="44" t="n">
+        <f aca="false">B28/B26</f>
+        <v>1.87119871033923</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="B30" s="40" t="n">
+        <f aca="false">('Kosten und Finanzierung'!B24+'Kosten und Finanzierung'!B25+'Kosten und Finanzierung'!B26)/B26</f>
+        <v>0.906538809168673</v>
+      </c>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="29" t="s">
+        <v>482</v>
+      </c>
+      <c r="B31" s="52" t="n">
+        <f aca="false">E19-B27</f>
+        <v>-1968261.72375817</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="B32" s="33" t="n">
+        <f aca="false">MAX(0,B28-0.8*B26)</f>
+        <v>2773890.03878097</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">E19/E5</f>
+        <v>17.1013032997038</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">B27/E5</f>
+        <v>28.7999430115732</v>
+      </c>
+      <c r="F34" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -4752,191 +4628,511 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>481</v>
+        <v>491</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>482</v>
+        <v>344</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>485</v>
+        <v>494</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>486</v>
-      </c>
-      <c r="B5" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>9610.17230350448</v>
-      </c>
-      <c r="C5" s="55" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B11/Tilgungsplan!N3</f>
-        <v>1.54192628304023</v>
-      </c>
-      <c r="D5" s="50"/>
+      <c r="A5" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="B5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(1-1)</f>
+        <v>87847.0588235294</v>
+      </c>
+      <c r="C5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(2-1)</f>
+        <v>89164.7647058823</v>
+      </c>
+      <c r="D5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(3-1)</f>
+        <v>90502.2361764706</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(4-1)</f>
+        <v>91859.7697191176</v>
+      </c>
+      <c r="F5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(5-1)</f>
+        <v>93237.6662649044</v>
+      </c>
+      <c r="G5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(6-1)</f>
+        <v>94636.2312588779</v>
+      </c>
+      <c r="H5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(7-1)</f>
+        <v>96055.7747277611</v>
+      </c>
+      <c r="I5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(8-1)</f>
+        <v>97496.6113486775</v>
+      </c>
+      <c r="J5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(9-1)</f>
+        <v>98959.0605189077</v>
+      </c>
+      <c r="K5" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$21*(1+Annahmen!$B$78)^(10-1)</f>
+        <v>100443.446426691</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>487</v>
-      </c>
-      <c r="B6" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-'Tilgung Jahre'!E14*0.01/12</f>
-        <v>6052.52203384148</v>
-      </c>
-      <c r="C6" s="55" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+'Tilgung Jahre'!E14*0.01/12)</f>
-        <v>1.2842759821744</v>
-      </c>
-      <c r="D6" s="50" t="n">
-        <f aca="false">B6-$B$5</f>
-        <v>-3557.650269663</v>
+        <v>503</v>
+      </c>
+      <c r="B6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(1-1)</f>
+        <v>19200</v>
+      </c>
+      <c r="C6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(2-1)</f>
+        <v>19584</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(3-1)</f>
+        <v>19975.68</v>
+      </c>
+      <c r="E6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(4-1)</f>
+        <v>20375.1936</v>
+      </c>
+      <c r="F6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(5-1)</f>
+        <v>20782.697472</v>
+      </c>
+      <c r="G6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(6-1)</f>
+        <v>21198.35142144</v>
+      </c>
+      <c r="H6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(7-1)</f>
+        <v>21622.3184498688</v>
+      </c>
+      <c r="I6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(8-1)</f>
+        <v>22054.7648188662</v>
+      </c>
+      <c r="J6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(9-1)</f>
+        <v>22495.8601152435</v>
+      </c>
+      <c r="K6" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$25*(1+Annahmen!$B$80)^(10-1)</f>
+        <v>22945.7773175484</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>488</v>
-      </c>
-      <c r="B7" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48)</f>
-        <v>8951.31936232801</v>
-      </c>
-      <c r="C7" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B11-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.50477297150681</v>
-      </c>
-      <c r="D7" s="50" t="n">
-        <f aca="false">B7-$B$5</f>
-        <v>-658.85294117647</v>
+        <v>380</v>
+      </c>
+      <c r="B7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(1-1)</f>
+        <v>61200</v>
+      </c>
+      <c r="C7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(2-1)</f>
+        <v>62118</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(3-1)</f>
+        <v>63049.77</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(4-1)</f>
+        <v>63995.51655</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(5-1)</f>
+        <v>64955.44929825</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(6-1)</f>
+        <v>65929.7810377237</v>
+      </c>
+      <c r="H7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(7-1)</f>
+        <v>66918.7277532896</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(8-1)</f>
+        <v>67922.5086695889</v>
+      </c>
+      <c r="J7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(9-1)</f>
+        <v>68941.3462996327</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <f aca="false">'Flächen und Mieten'!$G$22*(1+Annahmen!$B$78)^(10-1)</f>
+        <v>69975.4664941272</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>489</v>
+        <v>504</v>
       </c>
       <c r="B8" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-0.2*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>5645.17230350448</v>
-      </c>
-      <c r="C8" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B11-0.2*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.3183363572414</v>
+        <f aca="false">-Annahmen!$B$48*(B5+B6+B7)</f>
+        <v>-16824.7058823529</v>
+      </c>
+      <c r="C8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(C5+C6+C7)</f>
+        <v>-17086.6764705882</v>
       </c>
       <c r="D8" s="50" t="n">
-        <f aca="false">B8-$B$5</f>
-        <v>-3965</v>
+        <f aca="false">-Annahmen!$B$48*(D5+D6+D7)</f>
+        <v>-17352.7686176471</v>
+      </c>
+      <c r="E8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(E5+E6+E7)</f>
+        <v>-17623.0479869118</v>
+      </c>
+      <c r="F8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(F5+F6+F7)</f>
+        <v>-17897.5813035154</v>
+      </c>
+      <c r="G8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(G5+G6+G7)</f>
+        <v>-18176.4363718042</v>
+      </c>
+      <c r="H8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(H5+H6+H7)</f>
+        <v>-18459.6820930919</v>
+      </c>
+      <c r="I8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(I5+I6+I7)</f>
+        <v>-18747.3884837133</v>
+      </c>
+      <c r="J8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(J5+J6+J7)</f>
+        <v>-19039.6266933784</v>
+      </c>
+      <c r="K8" s="50" t="n">
+        <f aca="false">-Annahmen!$B$48*(K5+K6+K7)</f>
+        <v>-19336.4690238367</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="B9" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-0.4*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>1680.17230350448</v>
-      </c>
-      <c r="C9" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B11-0.4*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.09474643144258</v>
-      </c>
-      <c r="D9" s="50" t="n">
-        <f aca="false">B9-$B$5</f>
-        <v>-7930</v>
+        <v>385</v>
+      </c>
+      <c r="B9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(1-1))-B7-Annahmen!$B$51*12</f>
+        <v>288824.1</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(2-1))-C7-Annahmen!$B$51*12</f>
+        <v>293156.4615</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(3-1))-D7-Annahmen!$B$51*12</f>
+        <v>297553.8084225</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(4-1))-E7-Annahmen!$B$51*12</f>
+        <v>302017.115548837</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(5-1))-F7-Annahmen!$B$51*12</f>
+        <v>306547.37228207</v>
+      </c>
+      <c r="G9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(6-1))-G7-Annahmen!$B$51*12</f>
+        <v>311145.582866301</v>
+      </c>
+      <c r="H9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(7-1))-H7-Annahmen!$B$51*12</f>
+        <v>315812.766609295</v>
+      </c>
+      <c r="I9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(8-1))-I7-Annahmen!$B$51*12</f>
+        <v>320549.958108435</v>
+      </c>
+      <c r="J9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(9-1))-J7-Annahmen!$B$51*12</f>
+        <v>325358.207480061</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(10-1))-K7-Annahmen!$B$51*12</f>
+        <v>330238.580592262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>491</v>
-      </c>
-      <c r="B10" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12</f>
-        <v>8151.66258258539</v>
-      </c>
-      <c r="C10" s="55" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12)</f>
-        <v>1.4247456829052</v>
-      </c>
-      <c r="D10" s="50" t="n">
-        <f aca="false">B10-$B$5</f>
-        <v>-1458.50972091909</v>
+      <c r="A10" s="29" t="s">
+        <v>387</v>
+      </c>
+      <c r="B10" s="35" t="n">
+        <f aca="false">SUM(B5:B9)</f>
+        <v>440246.452941176</v>
+      </c>
+      <c r="C10" s="35" t="n">
+        <f aca="false">SUM(C5:C9)</f>
+        <v>446936.549735294</v>
+      </c>
+      <c r="D10" s="35" t="n">
+        <f aca="false">SUM(D5:D9)</f>
+        <v>453728.725981323</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <f aca="false">SUM(E5:E9)</f>
+        <v>460624.547431043</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <f aca="false">SUM(F5:F9)</f>
+        <v>467625.604013709</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <f aca="false">SUM(G5:G9)</f>
+        <v>474733.510212538</v>
+      </c>
+      <c r="H10" s="35" t="n">
+        <f aca="false">SUM(H5:H9)</f>
+        <v>481949.905447123</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <f aca="false">SUM(I5:I9)</f>
+        <v>489276.454461854</v>
+      </c>
+      <c r="J10" s="35" t="n">
+        <f aca="false">SUM(J5:J9)</f>
+        <v>496714.847720467</v>
+      </c>
+      <c r="K10" s="35" t="n">
+        <f aca="false">SUM(K5:K9)</f>
+        <v>504266.801806792</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>492</v>
+        <v>505</v>
       </c>
       <c r="B11" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-'Flächen und Mieten'!F23*(1-Annahmen!$B$48)</f>
-        <v>8755.17230350448</v>
-      </c>
-      <c r="C11" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B11-'Flächen und Mieten'!F23*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.49371206196633</v>
+        <f aca="false">-'Tilgung Jahre'!D5</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="C11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D6</f>
+        <v>-212800.285299123</v>
       </c>
       <c r="D11" s="50" t="n">
-        <f aca="false">B11-$B$5</f>
-        <v>-855</v>
+        <f aca="false">-'Tilgung Jahre'!D7</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="E11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D8</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="F11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D9</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="G11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D10</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="H11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D11</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="I11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D12</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="J11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D13</f>
+        <v>-212800.285299123</v>
+      </c>
+      <c r="K11" s="50" t="n">
+        <f aca="false">-'Tilgung Jahre'!D14</f>
+        <v>-212800.285299123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>493</v>
-      </c>
-      <c r="B12" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B13-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48)</f>
-        <v>8170.17230350448</v>
-      </c>
-      <c r="C12" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B11-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.46072338438946</v>
-      </c>
-      <c r="D12" s="50" t="n">
-        <f aca="false">B12-$B$5</f>
-        <v>-1440</v>
+      <c r="A12" s="29" t="s">
+        <v>506</v>
+      </c>
+      <c r="B12" s="52" t="n">
+        <f aca="false">B10+B11</f>
+        <v>227446.167642054</v>
+      </c>
+      <c r="C12" s="52" t="n">
+        <f aca="false">C10+C11</f>
+        <v>234136.264436171</v>
+      </c>
+      <c r="D12" s="52" t="n">
+        <f aca="false">D10+D11</f>
+        <v>240928.440682201</v>
+      </c>
+      <c r="E12" s="52" t="n">
+        <f aca="false">E10+E11</f>
+        <v>247824.26213192</v>
+      </c>
+      <c r="F12" s="52" t="n">
+        <f aca="false">F10+F11</f>
+        <v>254825.318714586</v>
+      </c>
+      <c r="G12" s="52" t="n">
+        <f aca="false">G10+G11</f>
+        <v>261933.224913416</v>
+      </c>
+      <c r="H12" s="52" t="n">
+        <f aca="false">H10+H11</f>
+        <v>269149.620148</v>
+      </c>
+      <c r="I12" s="52" t="n">
+        <f aca="false">I10+I11</f>
+        <v>276476.169162731</v>
+      </c>
+      <c r="J12" s="52" t="n">
+        <f aca="false">J10+J11</f>
+        <v>283914.562421344</v>
+      </c>
+      <c r="K12" s="52" t="n">
+        <f aca="false">K10+K11</f>
+        <v>291466.516507669</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>494</v>
-      </c>
-      <c r="B13" s="50" t="n">
-        <f aca="false">'Ertrag und Cashflow'!B9-'Ertrag und Cashflow'!B7*(1-Annahmen!$B$48)+'Ertrag und Cashflow'!B12</f>
-        <v>-9704.82769649552</v>
-      </c>
-      <c r="C13" s="55" t="n">
-        <f aca="false">('Ertrag und Cashflow'!B9-'Ertrag und Cashflow'!B7*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>0.45273601398491</v>
-      </c>
-      <c r="D13" s="50" t="n">
-        <f aca="false">B13-$B$5</f>
-        <v>-19315</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
-        <v>495</v>
+      <c r="A13" s="29" t="s">
+        <v>507</v>
+      </c>
+      <c r="B13" s="54" t="n">
+        <f aca="false">B10/-B11</f>
+        <v>2.06882454279769</v>
+      </c>
+      <c r="C13" s="54" t="n">
+        <f aca="false">C10/-C11</f>
+        <v>2.10026292543291</v>
+      </c>
+      <c r="D13" s="54" t="n">
+        <f aca="false">D10/-D11</f>
+        <v>2.13218100409753</v>
+      </c>
+      <c r="E13" s="54" t="n">
+        <f aca="false">E10/-E11</f>
+        <v>2.16458613663777</v>
+      </c>
+      <c r="F13" s="54" t="n">
+        <f aca="false">F10/-F11</f>
+        <v>2.19748579451569</v>
+      </c>
+      <c r="G13" s="54" t="n">
+        <f aca="false">G10/-G11</f>
+        <v>2.23088756457835</v>
+      </c>
+      <c r="H13" s="54" t="n">
+        <f aca="false">H10/-H11</f>
+        <v>2.26479915085485</v>
+      </c>
+      <c r="I13" s="54" t="n">
+        <f aca="false">I10/-I11</f>
+        <v>2.29922837638165</v>
+      </c>
+      <c r="J13" s="54" t="n">
+        <f aca="false">J10/-J11</f>
+        <v>2.33418318505663</v>
+      </c>
+      <c r="K13" s="54" t="n">
+        <f aca="false">K10/-K11</f>
+        <v>2.36967164352233</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="B14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E5</f>
+        <v>4796289.99144002</v>
+      </c>
+      <c r="C14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E6</f>
+        <v>4745376.85834322</v>
+      </c>
+      <c r="D14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E7</f>
+        <v>4692705.54860192</v>
+      </c>
+      <c r="E14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E8</f>
+        <v>4638213.05983898</v>
+      </c>
+      <c r="F14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E9</f>
+        <v>4581834.06036832</v>
+      </c>
+      <c r="G14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E10</f>
+        <v>4523500.80088865</v>
+      </c>
+      <c r="H14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E11</f>
+        <v>4463143.02276395</v>
+      </c>
+      <c r="I14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E12</f>
+        <v>4400687.86275702</v>
+      </c>
+      <c r="J14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E13</f>
+        <v>4336059.75407694</v>
+      </c>
+      <c r="K14" s="33" t="n">
+        <f aca="false">'Tilgung Jahre'!E14</f>
+        <v>4269180.3235956</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>508</v>
       </c>
     </row>
   </sheetData>
@@ -4956,338 +5152,191 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>496</v>
+        <v>509</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="43" t="s">
-        <v>498</v>
+        <v>510</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>499</v>
-      </c>
-      <c r="B4" s="19" t="n">
-        <v>90</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>500</v>
+      <c r="A4" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>501</v>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>600</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>502</v>
-      </c>
+      <c r="A5" s="29" t="s">
+        <v>515</v>
+      </c>
+      <c r="B5" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13</f>
+        <v>18953.8473035045</v>
+      </c>
+      <c r="C5" s="55" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B11/Tilgungsplan!N3</f>
+        <v>2.06882454279769</v>
+      </c>
+      <c r="D5" s="50"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>503</v>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>0.56</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>504</v>
+        <v>516</v>
+      </c>
+      <c r="B6" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-'Tilgung Jahre'!E14*0.01/12</f>
+        <v>15396.1970338415</v>
+      </c>
+      <c r="C6" s="55" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+'Tilgung Jahre'!E14*0.01/12)</f>
+        <v>1.72313144984421</v>
+      </c>
+      <c r="D6" s="50" t="n">
+        <f aca="false">B6-$B$5</f>
+        <v>-3557.650269663</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="B7" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>506</v>
+        <v>517</v>
+      </c>
+      <c r="B7" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48)</f>
+        <v>18294.994362328</v>
+      </c>
+      <c r="C7" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B11-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
+        <v>2.03167123126428</v>
+      </c>
+      <c r="D7" s="50" t="n">
+        <f aca="false">B7-$B$5</f>
+        <v>-658.852941176472</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>518</v>
+      </c>
+      <c r="B8" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-0.2*Annahmen!$B$49*Annahmen!$B$50</f>
+        <v>13120.1123035045</v>
+      </c>
+      <c r="C8" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B11-0.2*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
+        <v>1.73985496504737</v>
+      </c>
+      <c r="D8" s="50" t="n">
+        <f aca="false">B8-$B$5</f>
+        <v>-5833.735</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>509</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>233</v>
+      <c r="A9" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="B9" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-0.4*Annahmen!$B$49*Annahmen!$B$50</f>
+        <v>7286.37730350447</v>
+      </c>
+      <c r="C9" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B11-0.4*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
+        <v>1.41088538729705</v>
+      </c>
+      <c r="D9" s="50" t="n">
+        <f aca="false">B9-$B$5</f>
+        <v>-11667.47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>511</v>
-      </c>
-      <c r="B10" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="C10" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <v>60</v>
+        <v>520</v>
+      </c>
+      <c r="B10" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12</f>
+        <v>17495.3375825854</v>
+      </c>
+      <c r="C10" s="55" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12)</f>
+        <v>1.91160165596738</v>
+      </c>
+      <c r="D10" s="50" t="n">
+        <f aca="false">B10-$B$5</f>
+        <v>-1458.50972091909</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>512</v>
-      </c>
-      <c r="B11" s="20" t="n">
-        <v>0.174</v>
-      </c>
-      <c r="C11" s="20" t="n">
-        <v>0.362</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>513</v>
+        <v>521</v>
+      </c>
+      <c r="B11" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-'Flächen und Mieten'!F23*(1-Annahmen!$B$48)</f>
+        <v>18098.8473035045</v>
+      </c>
+      <c r="C11" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B11-'Flächen und Mieten'!F23*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
+        <v>2.0206103217238</v>
+      </c>
+      <c r="D11" s="50" t="n">
+        <f aca="false">B11-$B$5</f>
+        <v>-855</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>499</v>
-      </c>
-      <c r="B12" s="33" t="n">
-        <f aca="false">$B$4</f>
-        <v>90</v>
-      </c>
-      <c r="C12" s="33" t="n">
-        <f aca="false">$B$4</f>
-        <v>90</v>
-      </c>
-      <c r="D12" s="33" t="n">
-        <f aca="false">$B$4</f>
-        <v>90</v>
+        <v>522</v>
+      </c>
+      <c r="B12" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B13-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48)</f>
+        <v>17513.8473035045</v>
+      </c>
+      <c r="C12" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B11-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
+        <v>1.98762164414692</v>
+      </c>
+      <c r="D12" s="50" t="n">
+        <f aca="false">B12-$B$5</f>
+        <v>-1440</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>514</v>
-      </c>
-      <c r="B13" s="33" t="n">
-        <f aca="false">B12*365*B11/12</f>
-        <v>476.325</v>
-      </c>
-      <c r="C13" s="33" t="n">
-        <f aca="false">C12*365*C11/12</f>
-        <v>990.975</v>
-      </c>
-      <c r="D13" s="33" t="n">
-        <f aca="false">D12*365*D11/12</f>
-        <v>1642.5</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>515</v>
-      </c>
-      <c r="B14" s="33" t="n">
-        <f aca="false">B13*(1-$B$6)</f>
-        <v>209.583</v>
-      </c>
-      <c r="C14" s="33" t="n">
-        <f aca="false">C13*(1-$B$6)</f>
-        <v>436.029</v>
-      </c>
-      <c r="D14" s="33" t="n">
-        <f aca="false">D13*(1-$B$6)</f>
-        <v>722.7</v>
+        <v>523</v>
+      </c>
+      <c r="B13" s="50" t="n">
+        <f aca="false">'Ertrag und Cashflow'!B9-'Ertrag und Cashflow'!B7*(1-Annahmen!$B$48)+'Ertrag und Cashflow'!B12</f>
+        <v>-9704.82769649552</v>
+      </c>
+      <c r="C13" s="55" t="n">
+        <f aca="false">('Ertrag und Cashflow'!B9-'Ertrag und Cashflow'!B7*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
+        <v>0.45273601398491</v>
+      </c>
+      <c r="D13" s="50" t="n">
+        <f aca="false">B13-$B$5</f>
+        <v>-28658.675</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>516</v>
-      </c>
-      <c r="B15" s="33" t="n">
-        <f aca="false">B10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>603.529411764706</v>
-      </c>
-      <c r="C15" s="33" t="n">
-        <f aca="false">C10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>603.529411764706</v>
-      </c>
-      <c r="D15" s="33" t="n">
-        <f aca="false">D10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
-        <v>603.529411764706</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>518</v>
-      </c>
-      <c r="B16" s="33" t="n">
-        <f aca="false">B10*$B$5</f>
-        <v>36000</v>
-      </c>
-      <c r="C16" s="33" t="n">
-        <f aca="false">C10*$B$5</f>
-        <v>36000</v>
-      </c>
-      <c r="D16" s="33" t="n">
-        <f aca="false">D10*$B$5</f>
-        <v>36000</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>519</v>
-      </c>
-      <c r="B17" s="33" t="n">
-        <f aca="false">-B16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-150</v>
-      </c>
-      <c r="C17" s="33" t="n">
-        <f aca="false">-C16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-150</v>
-      </c>
-      <c r="D17" s="33" t="n">
-        <f aca="false">-D16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
-        <v>-150</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>520</v>
-      </c>
-      <c r="B18" s="52" t="n">
-        <f aca="false">B14-B15+B17</f>
-        <v>-543.946411764706</v>
-      </c>
-      <c r="C18" s="52" t="n">
-        <f aca="false">C14-C15+C17</f>
-        <v>-317.500411764706</v>
-      </c>
-      <c r="D18" s="52" t="n">
-        <f aca="false">D14-D15+D17</f>
-        <v>-30.8294117647059</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="s">
-        <v>521</v>
-      </c>
-      <c r="B19" s="51" t="n">
-        <f aca="false">B18</f>
-        <v>-543.946411764706</v>
-      </c>
-      <c r="C19" s="51" t="n">
-        <f aca="false">C18</f>
-        <v>-317.500411764706</v>
-      </c>
-      <c r="D19" s="51" t="n">
-        <f aca="false">D18</f>
-        <v>-30.8294117647059</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="s">
-        <v>522</v>
-      </c>
-      <c r="B20" s="29" t="str">
-        <f aca="false">IF(B19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
-        <v>lohnt sich nicht</v>
-      </c>
-      <c r="C20" s="29" t="str">
-        <f aca="false">IF(C19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
-        <v>lohnt sich nicht</v>
-      </c>
-      <c r="D20" s="29" t="str">
-        <f aca="false">IF(D19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
-        <v>lohnt sich nicht</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>523</v>
-      </c>
-      <c r="B21" s="40" t="n">
-        <f aca="false">(B15-B17)/(B12*365/12*(1-$B$6))</f>
-        <v>0.625595194491246</v>
-      </c>
-      <c r="C21" s="40" t="n">
-        <f aca="false">(C15-C17)/(C12*365/12*(1-$B$6))</f>
-        <v>0.625595194491246</v>
-      </c>
-      <c r="D21" s="40" t="n">
-        <f aca="false">(D15-D17)/(D12*365/12*(1-$B$6))</f>
-        <v>0.625595194491246</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="43" t="s">
+      <c r="A15" s="16" t="s">
         <v>524</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="43" t="str">
-        <f aca="false">IF(MAX(B19:D19)&gt;=B7,"Mindestens ein Szenario erreicht den Mindest-Mehrertrag: Airbnb prüfen.","Kein Szenario erreicht den Mindest-Mehrertrag von "&amp;TEXT(B7,"#,##0")&amp;" € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.")</f>
-        <v>Kein Szenario erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="43" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
-        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -5307,6 +5356,357 @@
     <tabColor rgb="FFC49A45"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="43" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>600</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>0.56</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>540</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="B12" s="33" t="n">
+        <f aca="false">$B$4</f>
+        <v>90</v>
+      </c>
+      <c r="C12" s="33" t="n">
+        <f aca="false">$B$4</f>
+        <v>90</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <f aca="false">$B$4</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="B13" s="33" t="n">
+        <f aca="false">B12*365*B11/12</f>
+        <v>476.325</v>
+      </c>
+      <c r="C13" s="33" t="n">
+        <f aca="false">C12*365*C11/12</f>
+        <v>990.975</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <f aca="false">D12*365*D11/12</f>
+        <v>1642.5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="B14" s="33" t="n">
+        <f aca="false">B13*(1-$B$6)</f>
+        <v>209.583</v>
+      </c>
+      <c r="C14" s="33" t="n">
+        <f aca="false">C13*(1-$B$6)</f>
+        <v>436.029</v>
+      </c>
+      <c r="D14" s="33" t="n">
+        <f aca="false">D13*(1-$B$6)</f>
+        <v>722.7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="B15" s="33" t="n">
+        <f aca="false">B10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
+        <v>603.529411764706</v>
+      </c>
+      <c r="C15" s="33" t="n">
+        <f aca="false">C10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
+        <v>603.529411764706</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <f aca="false">D10*Annahmen!$B$46*(1-Annahmen!$B$48)</f>
+        <v>603.529411764706</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>547</v>
+      </c>
+      <c r="B16" s="33" t="n">
+        <f aca="false">B10*$B$5</f>
+        <v>36000</v>
+      </c>
+      <c r="C16" s="33" t="n">
+        <f aca="false">C10*$B$5</f>
+        <v>36000</v>
+      </c>
+      <c r="D16" s="33" t="n">
+        <f aca="false">D10*$B$5</f>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>548</v>
+      </c>
+      <c r="B17" s="33" t="n">
+        <f aca="false">-B16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
+        <v>-150</v>
+      </c>
+      <c r="C17" s="33" t="n">
+        <f aca="false">-C16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
+        <v>-150</v>
+      </c>
+      <c r="D17" s="33" t="n">
+        <f aca="false">-D16*(Annahmen!$B$57+Annahmen!$B$58)/12</f>
+        <v>-150</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="B18" s="52" t="n">
+        <f aca="false">B14-B15+B17</f>
+        <v>-543.946411764706</v>
+      </c>
+      <c r="C18" s="52" t="n">
+        <f aca="false">C14-C15+C17</f>
+        <v>-317.500411764706</v>
+      </c>
+      <c r="D18" s="52" t="n">
+        <f aca="false">D14-D15+D17</f>
+        <v>-30.8294117647059</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="29" t="s">
+        <v>550</v>
+      </c>
+      <c r="B19" s="51" t="n">
+        <f aca="false">B18</f>
+        <v>-543.946411764706</v>
+      </c>
+      <c r="C19" s="51" t="n">
+        <f aca="false">C18</f>
+        <v>-317.500411764706</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <f aca="false">D18</f>
+        <v>-30.8294117647059</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="29" t="s">
+        <v>551</v>
+      </c>
+      <c r="B20" s="29" t="str">
+        <f aca="false">IF(B19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
+        <v>lohnt sich nicht</v>
+      </c>
+      <c r="C20" s="29" t="str">
+        <f aca="false">IF(C19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
+        <v>lohnt sich nicht</v>
+      </c>
+      <c r="D20" s="29" t="str">
+        <f aca="false">IF(D19&gt;=$B$7,"lohnt sich","lohnt sich nicht")</f>
+        <v>lohnt sich nicht</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="B21" s="40" t="n">
+        <f aca="false">(B15-B17)/(B12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+      <c r="C21" s="40" t="n">
+        <f aca="false">(C15-C17)/(C12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+      <c r="D21" s="40" t="n">
+        <f aca="false">(D15-D17)/(D12*365/12*(1-$B$6))</f>
+        <v>0.625595194491246</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="43" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="43" t="str">
+        <f aca="false">IF(MAX(B19:D19)&gt;=B7,"Mindestens ein Szenario erreicht den Mindest-Mehrertrag: Airbnb prüfen.","Kein Szenario erreicht den Mindest-Mehrertrag von "&amp;TEXT(B7,"#,##0")&amp;" € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.")</f>
+        <v>Kein Szenario erreicht den Mindest-Mehrertrag von 300 € pro Monat. Langfristige Vermietung ist besser, Airbnb bleibt aus dem Konzept.</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="16" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="43" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="16" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>560</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFC49A45"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5318,376 +5718,376 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>532</v>
+        <v>561</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>533</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>534</v>
+        <v>563</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>535</v>
+        <v>564</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>536</v>
+        <v>565</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>537</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="57" t="s">
-        <v>538</v>
-      </c>
-      <c r="C5" s="58" t="s">
-        <v>539</v>
-      </c>
-      <c r="D5" s="59" t="s">
-        <v>540</v>
+      <c r="B5" s="58" t="s">
+        <v>567</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>568</v>
+      </c>
+      <c r="D5" s="60" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="57" t="s">
-        <v>541</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>542</v>
-      </c>
-      <c r="D6" s="59" t="s">
-        <v>540</v>
+      <c r="B6" s="58" t="s">
+        <v>570</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>571</v>
+      </c>
+      <c r="D6" s="60" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="57" t="s">
-        <v>543</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>544</v>
-      </c>
-      <c r="D7" s="59" t="s">
-        <v>540</v>
+      <c r="B7" s="58" t="s">
+        <v>572</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>573</v>
+      </c>
+      <c r="D7" s="60" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="57" t="s">
-        <v>545</v>
-      </c>
-      <c r="C8" s="58" t="s">
-        <v>546</v>
-      </c>
-      <c r="D8" s="59" t="s">
-        <v>547</v>
+      <c r="B8" s="58" t="s">
+        <v>574</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>575</v>
+      </c>
+      <c r="D8" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="57" t="s">
-        <v>548</v>
-      </c>
-      <c r="C9" s="58" t="s">
-        <v>549</v>
-      </c>
-      <c r="D9" s="59" t="s">
-        <v>550</v>
+      <c r="B9" s="58" t="s">
+        <v>577</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>578</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>579</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="57" t="s">
-        <v>551</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>552</v>
-      </c>
-      <c r="D10" s="59" t="s">
-        <v>547</v>
+      <c r="B10" s="58" t="s">
+        <v>580</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>581</v>
+      </c>
+      <c r="D10" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="57" t="s">
-        <v>553</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>554</v>
-      </c>
-      <c r="D11" s="59" t="s">
-        <v>547</v>
+      <c r="B11" s="58" t="s">
+        <v>582</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>583</v>
+      </c>
+      <c r="D11" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="57" t="s">
-        <v>555</v>
-      </c>
-      <c r="C12" s="58" t="s">
-        <v>556</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>547</v>
+      <c r="B12" s="58" t="s">
+        <v>584</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>585</v>
+      </c>
+      <c r="D12" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="28" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="57" t="s">
-        <v>557</v>
-      </c>
-      <c r="C13" s="58" t="s">
-        <v>558</v>
-      </c>
-      <c r="D13" s="59" t="s">
-        <v>547</v>
+      <c r="B13" s="58" t="s">
+        <v>586</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>587</v>
+      </c>
+      <c r="D13" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="57" t="s">
-        <v>559</v>
-      </c>
-      <c r="C14" s="58" t="s">
-        <v>560</v>
-      </c>
-      <c r="D14" s="59" t="s">
-        <v>547</v>
+      <c r="B14" s="58" t="s">
+        <v>588</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>589</v>
+      </c>
+      <c r="D14" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="57" t="s">
-        <v>561</v>
-      </c>
-      <c r="C15" s="58" t="s">
-        <v>562</v>
-      </c>
-      <c r="D15" s="59" t="s">
-        <v>540</v>
+      <c r="B15" s="58" t="s">
+        <v>590</v>
+      </c>
+      <c r="C15" s="59" t="s">
+        <v>591</v>
+      </c>
+      <c r="D15" s="60" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="57" t="s">
-        <v>563</v>
-      </c>
-      <c r="C16" s="58" t="s">
-        <v>564</v>
-      </c>
-      <c r="D16" s="59" t="s">
-        <v>547</v>
+      <c r="B16" s="58" t="s">
+        <v>592</v>
+      </c>
+      <c r="C16" s="59" t="s">
+        <v>593</v>
+      </c>
+      <c r="D16" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="57" t="s">
-        <v>565</v>
-      </c>
-      <c r="C17" s="58" t="s">
-        <v>566</v>
-      </c>
-      <c r="D17" s="59" t="s">
-        <v>547</v>
+      <c r="B17" s="58" t="s">
+        <v>594</v>
+      </c>
+      <c r="C17" s="59" t="s">
+        <v>595</v>
+      </c>
+      <c r="D17" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="57" t="s">
-        <v>567</v>
-      </c>
-      <c r="C18" s="58" t="s">
-        <v>568</v>
-      </c>
-      <c r="D18" s="59" t="s">
-        <v>547</v>
+      <c r="B18" s="58" t="s">
+        <v>596</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>597</v>
+      </c>
+      <c r="D18" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="28" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="58" t="s">
+        <v>598</v>
+      </c>
+      <c r="C19" s="59" t="s">
+        <v>599</v>
+      </c>
+      <c r="D19" s="60" t="s">
         <v>569</v>
-      </c>
-      <c r="C19" s="58" t="s">
-        <v>570</v>
-      </c>
-      <c r="D19" s="59" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="28" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="57" t="s">
-        <v>571</v>
-      </c>
-      <c r="C20" s="58" t="s">
-        <v>572</v>
-      </c>
-      <c r="D20" s="59" t="s">
-        <v>547</v>
+      <c r="B20" s="58" t="s">
+        <v>600</v>
+      </c>
+      <c r="C20" s="59" t="s">
+        <v>601</v>
+      </c>
+      <c r="D20" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="57" t="s">
-        <v>573</v>
-      </c>
-      <c r="C21" s="58" t="s">
-        <v>574</v>
-      </c>
-      <c r="D21" s="59" t="s">
-        <v>547</v>
+      <c r="B21" s="58" t="s">
+        <v>602</v>
+      </c>
+      <c r="C21" s="59" t="s">
+        <v>603</v>
+      </c>
+      <c r="D21" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="57" t="s">
-        <v>575</v>
-      </c>
-      <c r="C22" s="58" t="s">
+      <c r="B22" s="58" t="s">
+        <v>604</v>
+      </c>
+      <c r="C22" s="59" t="s">
+        <v>605</v>
+      </c>
+      <c r="D22" s="60" t="s">
         <v>576</v>
-      </c>
-      <c r="D22" s="59" t="s">
-        <v>547</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="57" t="s">
-        <v>577</v>
-      </c>
-      <c r="C23" s="58" t="s">
-        <v>578</v>
-      </c>
-      <c r="D23" s="59" t="s">
-        <v>540</v>
+      <c r="B23" s="58" t="s">
+        <v>606</v>
+      </c>
+      <c r="C23" s="59" t="s">
+        <v>607</v>
+      </c>
+      <c r="D23" s="60" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="57" t="s">
-        <v>579</v>
-      </c>
-      <c r="C24" s="58" t="s">
-        <v>580</v>
-      </c>
-      <c r="D24" s="59" t="s">
-        <v>547</v>
+      <c r="B24" s="58" t="s">
+        <v>608</v>
+      </c>
+      <c r="C24" s="59" t="s">
+        <v>609</v>
+      </c>
+      <c r="D24" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="57" t="s">
-        <v>581</v>
-      </c>
-      <c r="C25" s="58" t="s">
-        <v>582</v>
-      </c>
-      <c r="D25" s="59" t="s">
-        <v>547</v>
+      <c r="B25" s="58" t="s">
+        <v>610</v>
+      </c>
+      <c r="C25" s="59" t="s">
+        <v>611</v>
+      </c>
+      <c r="D25" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="57" t="s">
-        <v>583</v>
-      </c>
-      <c r="C26" s="58" t="s">
-        <v>584</v>
-      </c>
-      <c r="D26" s="59" t="s">
-        <v>547</v>
+      <c r="B26" s="58" t="s">
+        <v>612</v>
+      </c>
+      <c r="C26" s="59" t="s">
+        <v>613</v>
+      </c>
+      <c r="D26" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="28" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="57" t="s">
-        <v>585</v>
-      </c>
-      <c r="C27" s="58" t="s">
-        <v>586</v>
-      </c>
-      <c r="D27" s="59" t="s">
-        <v>547</v>
+      <c r="B27" s="58" t="s">
+        <v>614</v>
+      </c>
+      <c r="C27" s="59" t="s">
+        <v>615</v>
+      </c>
+      <c r="D27" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="57" t="s">
-        <v>587</v>
-      </c>
-      <c r="C28" s="58" t="s">
-        <v>588</v>
-      </c>
-      <c r="D28" s="59" t="s">
-        <v>547</v>
+      <c r="B28" s="58" t="s">
+        <v>616</v>
+      </c>
+      <c r="C28" s="59" t="s">
+        <v>617</v>
+      </c>
+      <c r="D28" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="28" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="57" t="s">
-        <v>589</v>
-      </c>
-      <c r="C29" s="58" t="s">
-        <v>590</v>
-      </c>
-      <c r="D29" s="59" t="s">
-        <v>547</v>
+      <c r="B29" s="58" t="s">
+        <v>618</v>
+      </c>
+      <c r="C29" s="59" t="s">
+        <v>619</v>
+      </c>
+      <c r="D29" s="60" t="s">
+        <v>576</v>
       </c>
     </row>
   </sheetData>
@@ -6211,7 +6611,8 @@
         <v>135</v>
       </c>
       <c r="B49" s="21" t="n">
-        <v>65000</v>
+        <f aca="false">'Gastro Tagesteile'!F14</f>
+        <v>95635</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>136</v>
@@ -7317,7 +7718,7 @@
       </c>
       <c r="D17" s="33" t="n">
         <f aca="false">Annahmen!$B$49*12/D15</f>
-        <v>4105.26315789474</v>
+        <v>6040.1052631579</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>250</v>
@@ -7329,7 +7730,7 @@
       </c>
       <c r="D18" s="40" t="n">
         <f aca="false">'Flächen und Mieten'!F22/Annahmen!$B$49</f>
-        <v>0.0784615384615385</v>
+        <v>0.0533277565744759</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>252</v>
@@ -36688,11 +37089,11 @@
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">'Gastro Betrieb'!C19</f>
-        <v>14725</v>
+        <v>24068.675</v>
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">B10*12</f>
-        <v>176700</v>
+        <v>288824.1</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>386</v>
@@ -36704,11 +37105,11 @@
       </c>
       <c r="B11" s="35" t="n">
         <f aca="false">B9+B10</f>
-        <v>27343.5294117647</v>
+        <v>36687.2044117647</v>
       </c>
       <c r="C11" s="35" t="n">
         <f aca="false">B11*12</f>
-        <v>328122.352941177</v>
+        <v>440246.452941176</v>
       </c>
       <c r="D11" s="9"/>
     </row>
@@ -36732,11 +37133,11 @@
       </c>
       <c r="B13" s="51" t="n">
         <f aca="false">B11+B12</f>
-        <v>9610.17230350448</v>
+        <v>18953.8473035045</v>
       </c>
       <c r="C13" s="52" t="n">
         <f aca="false">B13*12</f>
-        <v>115322.067642054</v>
+        <v>227446.167642054</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>389</v>
@@ -36748,7 +37149,7 @@
       </c>
       <c r="B15" s="53" t="n">
         <f aca="false">B11/-B12</f>
-        <v>1.54192628304023</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>40</v>
@@ -36784,7 +37185,7 @@
       </c>
       <c r="B18" s="55" t="n">
         <f aca="false">B11/('Tilgung Jahre'!B5/12)</f>
-        <v>2.00582702527136</v>
+        <v>2.69124680221824</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Gastro-Konzept: Frühstück und Bowls tagsüber, abends Bar mit Snacks; Umsatzmodell, Flächen, Personal angepasst
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJGZfxHv7bzYyqdLwg8aFJ
</commit_message>
<xml_diff>
--- a/praesentation/Bankunterlagen_Baufeld3.xlsx
+++ b/praesentation/Bankunterlagen_Baufeld3.xlsx
@@ -397,13 +397,13 @@
     <t xml:space="preserve">Bar- und Theken-Zone (m²)</t>
   </si>
   <si>
-    <t xml:space="preserve">Theke, Backbar, Service</t>
+    <t xml:space="preserve">große Theke, Backbar, Service, Stehtische (Bar im Fokus)</t>
   </si>
   <si>
     <t xml:space="preserve">Küche mit Spülküche (m²)</t>
   </si>
   <si>
-    <t xml:space="preserve">Richtwert ca. 25–30 % der Gastraumfläche</t>
+    <t xml:space="preserve">kleine Bowl- und Snack-Küche, keine große Restaurantküche</t>
   </si>
   <si>
     <t xml:space="preserve">Lager, Kühlung, Anlieferung (m²)</t>
@@ -754,7 +754,7 @@
     <t xml:space="preserve">Bar und Theken-Zone</t>
   </si>
   <si>
-    <t xml:space="preserve">Küche mit Spülküche</t>
+    <t xml:space="preserve">Küche (Bowls, Snacks) mit Spülküche</t>
   </si>
   <si>
     <t xml:space="preserve">Lager, Kühlung, Anlieferung</t>
@@ -1303,10 +1303,10 @@
     <t xml:space="preserve">Bei sehr niedrigem Umsatz drücken Fixkosten stärker: die Rechnung ist dort zu günstig.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastro-Umsatz nach Tagesteilen: Frühstück, Mittag, Abend, Bar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hauptfokus Abend mit Restaurant und Bar. Öffnungstage, Gäste und Bon sind Annahmen (keine Marktdaten für Werlte), Ruhetag Montag.</t>
+    <t xml:space="preserve">Gastro-Umsatz nach Tagesteilen: Frühstück, Mittag, Bar am Abend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tagsüber Frühstück und Bowls, abends Bar mit Snacks. Öffnungstage, Gäste und Bon sind Annahmen (keine Marktdaten für Werlte), Ruhetag Montag.</t>
   </si>
   <si>
     <t xml:space="preserve">Tagesteil</t>
@@ -1339,31 +1339,31 @@
     <t xml:space="preserve">Sa, So 09:00–14:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Mittagstisch</t>
+    <t xml:space="preserve">Mittag: Bowls, Salate, Suppe</t>
   </si>
   <si>
     <t xml:space="preserve">Di–Fr 11:30–14:30</t>
   </si>
   <si>
-    <t xml:space="preserve">Abendessen Restaurant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Di–So 17:30–22:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bar Di–Do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ab 21:00</t>
+    <t xml:space="preserve">Nachmittag: Kaffee, Kuchen, Snacks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di–So 14:30–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar mit Snacks Di–Do, So</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ab 17:00</t>
   </si>
   <si>
     <t xml:space="preserve">Bar Fr, Sa (bis 01:00)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cocktails, Wein, Bier, Musik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feiern, Live-Abende, Séparée</t>
+    <t xml:space="preserve">Cocktails, Wein, Bier, Snacks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events: Live-Musik, Feiern</t>
   </si>
   <si>
     <t xml:space="preserve">nach Absprache, 4 pro Monat</t>
@@ -1372,10 +1372,10 @@
     <t xml:space="preserve">Gastro-Umsatz pro Monat (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">davon Tag (Frühstück, Brunch, Mittag)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">davon Abend (Restaurant, Bar, Feiern)</t>
+    <t xml:space="preserve">davon Tag (Frühstück, Brunch, Mittag, Nachmittag)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">davon Abend (Bar mit Snacks, Events)</t>
   </si>
   <si>
     <t xml:space="preserve">Gäste pro Monat</t>
@@ -1384,10 +1384,10 @@
     <t xml:space="preserve">Umsatz je Platz und Jahr (190 Plätze)</t>
   </si>
   <si>
-    <t xml:space="preserve">Auslastung der Plätze am Abend (Restaurantgäste je Tag / Plätze)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einordnung: Der Abend (Restaurant, Bar, Feiern) trägt den größten Teil des Umsatzes, Frühstück und Mittagstisch füllen das Haus am Tag. Terrasse im Sommer, Catering und Weihnachtsfeiern sind nicht eingerechnet. Branchen-Median Österreich ca. 12.000 € je Platz und Jahr.</t>
+    <t xml:space="preserve">Auslastung der Plätze an der Bar Fr, Sa (Gäste je Abend / Plätze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einordnung: Die Bar mit Snacks am Abend trägt den größten Teil des Umsatzes, Frühstück und Bowls füllen das Haus am Tag. Terrasse im Sommer, Catering und Weihnachtsfeiern sind nicht eingerechnet. Branchen-Median Österreich ca. 12.000 € je Platz und Jahr.</t>
   </si>
   <si>
     <t xml:space="preserve">Ertragswert und Beleihung</t>
@@ -1756,7 +1756,7 @@
     <t xml:space="preserve">Projekt: Gastro-Konzept mit Gestaltung</t>
   </si>
   <si>
-    <t xml:space="preserve">Konzept, Grundriss, Speisekarte, Umsatzaufbau.</t>
+    <t xml:space="preserve">Konzept (Frühstück, Bowls, Bar mit Snacks), Grundriss, Karte, Umsatzaufbau.</t>
   </si>
   <si>
     <t xml:space="preserve">Projekt: Lageplan, Flurkarte, Grundbuchauszug</t>
@@ -2743,11 +2743,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="85622033"/>
-        <c:axId val="35587217"/>
+        <c:axId val="88830755"/>
+        <c:axId val="14380942"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="85622033"/>
+        <c:axId val="88830755"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2813,7 +2813,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35587217"/>
+        <c:crossAx val="14380942"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2821,7 +2821,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="35587217"/>
+        <c:axId val="14380942"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2897,7 +2897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85622033"/>
+        <c:crossAx val="88830755"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">'Ertrag und Cashflow'!B10</f>
-        <v>24068.675</v>
+        <v>14728.05</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>37</v>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>18953.8473035045</v>
+        <v>9613.22230350448</v>
       </c>
       <c r="C25" s="9"/>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">'Ertrag und Cashflow'!B15</f>
-        <v>2.06882454279769</v>
+        <v>1.54209827529084</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>40</v>
@@ -3542,7 +3542,7 @@
       <c r="B5" s="7"/>
       <c r="C5" s="10" t="n">
         <f aca="false">Annahmen!$B$49</f>
-        <v>95635</v>
+        <v>65010</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="C6" s="33" t="n">
         <f aca="false">-$C$5*B6</f>
-        <v>-26777.8</v>
+        <v>-18202.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="C7" s="33" t="n">
         <f aca="false">-$C$5*B7</f>
-        <v>-28690.5</v>
+        <v>-19503</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="C8" s="33" t="n">
         <f aca="false">-$C$5*B8</f>
-        <v>-2869.05</v>
+        <v>-1950.3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C9" s="33" t="n">
         <f aca="false">-$C$5*B9</f>
-        <v>-1912.7</v>
+        <v>-1300.2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">-$C$5*B10</f>
-        <v>-1434.525</v>
+        <v>-975.15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C11" s="33" t="n">
         <f aca="false">-$C$5*B11</f>
-        <v>-1434.525</v>
+        <v>-975.15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">-$C$5*B12</f>
-        <v>-1434.525</v>
+        <v>-975.15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">-$C$5*B13</f>
-        <v>-956.35</v>
+        <v>-650.1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">-$C$5*B14</f>
-        <v>-956.35</v>
+        <v>-650.1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="C15" s="35" t="n">
         <f aca="false">SUM(C6:C14)</f>
-        <v>-66466.325</v>
+        <v>-45181.95</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="C16" s="35" t="n">
         <f aca="false">C5+C15</f>
-        <v>29168.675</v>
+        <v>19828.05</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>414</v>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C19" s="46" t="n">
         <f aca="false">C16+C17+C18</f>
-        <v>24068.675</v>
+        <v>14728.05</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3732,68 +3732,68 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="C24" s="33" t="n">
         <f aca="false">A24*$B$16</f>
-        <v>15250</v>
+        <v>12200</v>
       </c>
       <c r="D24" s="50" t="n">
         <f aca="false">C24-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>10150</v>
+        <v>7100</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="n">
-        <v>65000</v>
+        <v>50000</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">A25*$B$16</f>
-        <v>19825</v>
+        <v>15250</v>
       </c>
       <c r="D25" s="50" t="n">
         <f aca="false">C25-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>14725</v>
+        <v>10150</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="n">
-        <v>80000</v>
+        <f aca="false">Annahmen!$B$49</f>
+        <v>65010</v>
       </c>
       <c r="C26" s="33" t="n">
         <f aca="false">A26*$B$16</f>
-        <v>24400</v>
+        <v>19828.05</v>
       </c>
       <c r="D26" s="50" t="n">
         <f aca="false">C26-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>19300</v>
+        <v>14728.05</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="n">
-        <f aca="false">Annahmen!$B$49</f>
-        <v>95635</v>
+        <v>80000</v>
       </c>
       <c r="C27" s="33" t="n">
         <f aca="false">A27*$B$16</f>
-        <v>29168.675</v>
+        <v>24400</v>
       </c>
       <c r="D27" s="50" t="n">
         <f aca="false">C27-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>24068.675</v>
+        <v>19300</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="n">
-        <v>110000</v>
+        <v>95000</v>
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">A28*$B$16</f>
-        <v>33550</v>
+        <v>28975</v>
       </c>
       <c r="D28" s="50" t="n">
         <f aca="false">C28-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>28450</v>
+        <v>23875</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,18 +3872,18 @@
         <v>17</v>
       </c>
       <c r="D5" s="57" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>11</v>
       </c>
       <c r="F5" s="33" t="n">
         <f aca="false">C5*D5*E5</f>
-        <v>4675</v>
+        <v>5610</v>
       </c>
       <c r="G5" s="40" t="n">
         <f aca="false">F5/$F$14</f>
-        <v>0.0488837768599362</v>
+        <v>0.0862944162436548</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="G6" s="40" t="n">
         <f aca="false">F6/$F$14</f>
-        <v>0.0790505568045172</v>
+        <v>0.116289801568989</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3922,18 +3922,18 @@
         <v>17</v>
       </c>
       <c r="D7" s="57" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F7" s="33" t="n">
         <f aca="false">C7*D7*E7</f>
-        <v>11900</v>
+        <v>8840</v>
       </c>
       <c r="G7" s="40" t="n">
         <f aca="false">F7/$F$14</f>
-        <v>0.12443143200711</v>
+        <v>0.135979080141517</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,18 +3947,18 @@
         <v>26</v>
       </c>
       <c r="D8" s="57" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="F8" s="33" t="n">
         <f aca="false">C8*D8*E8</f>
-        <v>45760</v>
+        <v>3640</v>
       </c>
       <c r="G8" s="40" t="n">
         <f aca="false">F8/$F$14</f>
-        <v>0.478485909970199</v>
+        <v>0.0559913859406245</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,21 +3969,21 @@
         <v>439</v>
       </c>
       <c r="C9" s="57" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D9" s="57" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>20</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>18</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">C9*D9*E9</f>
-        <v>4680</v>
+        <v>11900</v>
       </c>
       <c r="G9" s="40" t="n">
         <f aca="false">F9/$F$14</f>
-        <v>0.0489360589742249</v>
+        <v>0.183048761728965</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3997,18 +3997,18 @@
         <v>9</v>
       </c>
       <c r="D10" s="57" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F10" s="33" t="n">
         <f aca="false">C10*D10*E10</f>
-        <v>13860</v>
+        <v>21060</v>
       </c>
       <c r="G10" s="40" t="n">
         <f aca="false">F10/$F$14</f>
-        <v>0.144926020808281</v>
+        <v>0.323950161513613</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,15 +4025,15 @@
         <v>40</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F11" s="33" t="n">
         <f aca="false">C11*D11*E11</f>
-        <v>7200</v>
+        <v>6400</v>
       </c>
       <c r="G11" s="40" t="n">
         <f aca="false">F11/$F$14</f>
-        <v>0.0752862445757307</v>
+        <v>0.0984463928626365</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F14" s="46" t="n">
         <f aca="false">SUM(F5:F11)</f>
-        <v>95635</v>
+        <v>65010</v>
       </c>
       <c r="G14" s="42" t="n">
         <f aca="false">SUM(G5:G11)</f>
@@ -4054,12 +4054,12 @@
         <v>445</v>
       </c>
       <c r="F15" s="33" t="n">
-        <f aca="false">SUM(F5:F7)</f>
-        <v>24135</v>
+        <f aca="false">SUM(F5:F8)</f>
+        <v>25650</v>
       </c>
       <c r="G15" s="40" t="n">
         <f aca="false">F15/F14</f>
-        <v>0.252365765671564</v>
+        <v>0.394554683894785</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,12 +4067,12 @@
         <v>446</v>
       </c>
       <c r="F16" s="35" t="n">
-        <f aca="false">SUM(F8:F11)</f>
-        <v>71500</v>
+        <f aca="false">SUM(F9:F11)</f>
+        <v>39360</v>
       </c>
       <c r="G16" s="42" t="n">
         <f aca="false">F16/F14</f>
-        <v>0.747634234328436</v>
+        <v>0.605445316105215</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="F17" s="28" t="n">
         <f aca="false">SUMPRODUCT(C5:C11,D5:D11)</f>
-        <v>4295</v>
+        <v>3815</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="F18" s="33" t="n">
         <f aca="false">F14*12/(Annahmen!$B$36+Annahmen!$B$37)</f>
-        <v>6040.1052631579</v>
+        <v>4105.89473684211</v>
       </c>
       <c r="G18" s="9"/>
     </row>
@@ -4099,8 +4099,8 @@
         <v>449</v>
       </c>
       <c r="F19" s="40" t="n">
-        <f aca="false">D8/(Annahmen!$B$36+Annahmen!$B$37)</f>
-        <v>0.289473684210526</v>
+        <f aca="false">D10/(Annahmen!$B$36+Annahmen!$B$37)</f>
+        <v>0.473684210526316</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4866,43 +4866,43 @@
       </c>
       <c r="B9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(1-1))-B7-Annahmen!$B$51*12</f>
-        <v>288824.1</v>
+        <v>176736.6</v>
       </c>
       <c r="C9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(2-1))-C7-Annahmen!$B$51*12</f>
-        <v>293156.4615</v>
+        <v>179387.649</v>
       </c>
       <c r="D9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(3-1))-D7-Annahmen!$B$51*12</f>
-        <v>297553.8084225</v>
+        <v>182078.463735</v>
       </c>
       <c r="E9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(4-1))-E7-Annahmen!$B$51*12</f>
-        <v>302017.115548837</v>
+        <v>184809.640691025</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(5-1))-F7-Annahmen!$B$51*12</f>
-        <v>306547.37228207</v>
+        <v>187581.78530139</v>
       </c>
       <c r="G9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(6-1))-G7-Annahmen!$B$51*12</f>
-        <v>311145.582866301</v>
+        <v>190395.512080911</v>
       </c>
       <c r="H9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(7-1))-H7-Annahmen!$B$51*12</f>
-        <v>315812.766609295</v>
+        <v>193251.444762125</v>
       </c>
       <c r="I9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(8-1))-I7-Annahmen!$B$51*12</f>
-        <v>320549.958108435</v>
+        <v>196150.216433557</v>
       </c>
       <c r="J9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(9-1))-J7-Annahmen!$B$51*12</f>
-        <v>325358.207480061</v>
+        <v>199092.46968006</v>
       </c>
       <c r="K9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(10-1))-K7-Annahmen!$B$51*12</f>
-        <v>330238.580592262</v>
+        <v>202078.856725261</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4911,43 +4911,43 @@
       </c>
       <c r="B10" s="35" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>440246.452941176</v>
+        <v>328158.952941176</v>
       </c>
       <c r="C10" s="35" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>446936.549735294</v>
+        <v>333167.737235294</v>
       </c>
       <c r="D10" s="35" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>453728.725981323</v>
+        <v>338253.381293823</v>
       </c>
       <c r="E10" s="35" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>460624.547431043</v>
+        <v>343417.072573231</v>
       </c>
       <c r="F10" s="35" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>467625.604013709</v>
+        <v>348660.017033029</v>
       </c>
       <c r="G10" s="35" t="n">
         <f aca="false">SUM(G5:G9)</f>
-        <v>474733.510212538</v>
+        <v>353983.439427149</v>
       </c>
       <c r="H10" s="35" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>481949.905447123</v>
+        <v>359388.583599952</v>
       </c>
       <c r="I10" s="35" t="n">
         <f aca="false">SUM(I5:I9)</f>
-        <v>489276.454461854</v>
+        <v>364876.712786976</v>
       </c>
       <c r="J10" s="35" t="n">
         <f aca="false">SUM(J5:J9)</f>
-        <v>496714.847720467</v>
+        <v>370449.109920465</v>
       </c>
       <c r="K10" s="35" t="n">
         <f aca="false">SUM(K5:K9)</f>
-        <v>504266.801806792</v>
+        <v>376107.077939791</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5001,43 +5001,43 @@
       </c>
       <c r="B12" s="52" t="n">
         <f aca="false">B10+B11</f>
-        <v>227446.167642054</v>
+        <v>115358.667642054</v>
       </c>
       <c r="C12" s="52" t="n">
         <f aca="false">C10+C11</f>
-        <v>234136.264436171</v>
+        <v>120367.451936171</v>
       </c>
       <c r="D12" s="52" t="n">
         <f aca="false">D10+D11</f>
-        <v>240928.440682201</v>
+        <v>125453.095994701</v>
       </c>
       <c r="E12" s="52" t="n">
         <f aca="false">E10+E11</f>
-        <v>247824.26213192</v>
+        <v>130616.787274108</v>
       </c>
       <c r="F12" s="52" t="n">
         <f aca="false">F10+F11</f>
-        <v>254825.318714586</v>
+        <v>135859.731733907</v>
       </c>
       <c r="G12" s="52" t="n">
         <f aca="false">G10+G11</f>
-        <v>261933.224913416</v>
+        <v>141183.154128026</v>
       </c>
       <c r="H12" s="52" t="n">
         <f aca="false">H10+H11</f>
-        <v>269149.620148</v>
+        <v>146588.298300829</v>
       </c>
       <c r="I12" s="52" t="n">
         <f aca="false">I10+I11</f>
-        <v>276476.169162731</v>
+        <v>152076.427487853</v>
       </c>
       <c r="J12" s="52" t="n">
         <f aca="false">J10+J11</f>
-        <v>283914.562421344</v>
+        <v>157648.824621343</v>
       </c>
       <c r="K12" s="52" t="n">
         <f aca="false">K10+K11</f>
-        <v>291466.516507669</v>
+        <v>163306.792640668</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5046,43 +5046,43 @@
       </c>
       <c r="B13" s="54" t="n">
         <f aca="false">B10/-B11</f>
-        <v>2.06882454279769</v>
+        <v>1.54209827529084</v>
       </c>
       <c r="C13" s="54" t="n">
         <f aca="false">C10/-C11</f>
-        <v>2.10026292543291</v>
+        <v>1.56563576391346</v>
       </c>
       <c r="D13" s="54" t="n">
         <f aca="false">D10/-D11</f>
-        <v>2.13218100409753</v>
+        <v>1.58953443515528</v>
       </c>
       <c r="E13" s="54" t="n">
         <f aca="false">E10/-E11</f>
-        <v>2.16458613663777</v>
+        <v>1.61379986916139</v>
       </c>
       <c r="F13" s="54" t="n">
         <f aca="false">F10/-F11</f>
-        <v>2.19748579451569</v>
+        <v>1.63843773302717</v>
       </c>
       <c r="G13" s="54" t="n">
         <f aca="false">G10/-G11</f>
-        <v>2.23088756457835</v>
+        <v>1.6634537821675</v>
       </c>
       <c r="H13" s="54" t="n">
         <f aca="false">H10/-H11</f>
-        <v>2.26479915085485</v>
+        <v>1.68885386170783</v>
       </c>
       <c r="I13" s="54" t="n">
         <f aca="false">I10/-I11</f>
-        <v>2.29922837638165</v>
+        <v>1.71464390789743</v>
       </c>
       <c r="J13" s="54" t="n">
         <f aca="false">J10/-J11</f>
-        <v>2.33418318505663</v>
+        <v>1.74082994954515</v>
       </c>
       <c r="K13" s="54" t="n">
         <f aca="false">K10/-K11</f>
-        <v>2.36967164352233</v>
+        <v>1.76741810947817</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5190,11 +5190,11 @@
       </c>
       <c r="B5" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>18953.8473035045</v>
+        <v>9613.22230350448</v>
       </c>
       <c r="C5" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/Tilgungsplan!N3</f>
-        <v>2.06882454279769</v>
+        <v>1.54209827529084</v>
       </c>
       <c r="D5" s="50"/>
     </row>
@@ -5204,11 +5204,11 @@
       </c>
       <c r="B6" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Tilgung Jahre'!E14*0.01/12</f>
-        <v>15396.1970338415</v>
+        <v>6055.57203384148</v>
       </c>
       <c r="C6" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+'Tilgung Jahre'!E14*0.01/12)</f>
-        <v>1.72313144984421</v>
+        <v>1.28441923514246</v>
       </c>
       <c r="D6" s="50" t="n">
         <f aca="false">B6-$B$5</f>
@@ -5221,15 +5221,15 @@
       </c>
       <c r="B7" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48)</f>
-        <v>18294.994362328</v>
+        <v>8954.36936232801</v>
       </c>
       <c r="C7" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>2.03167123126428</v>
+        <v>1.50494496375743</v>
       </c>
       <c r="D7" s="50" t="n">
         <f aca="false">B7-$B$5</f>
-        <v>-658.852941176472</v>
+        <v>-658.85294117647</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,15 +5238,15 @@
       </c>
       <c r="B8" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.2*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>13120.1123035045</v>
+        <v>5647.61230350448</v>
       </c>
       <c r="C8" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.2*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.73985496504737</v>
+        <v>1.31847395104189</v>
       </c>
       <c r="D8" s="50" t="n">
         <f aca="false">B8-$B$5</f>
-        <v>-5833.735</v>
+        <v>-3965.61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5255,15 +5255,15 @@
       </c>
       <c r="B9" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.4*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>7286.37730350447</v>
+        <v>1682.00230350448</v>
       </c>
       <c r="C9" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.4*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.41088538729705</v>
+        <v>1.09484962679294</v>
       </c>
       <c r="D9" s="50" t="n">
         <f aca="false">B9-$B$5</f>
-        <v>-11667.47</v>
+        <v>-7931.22</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5272,11 +5272,11 @@
       </c>
       <c r="B10" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12</f>
-        <v>17495.3375825854</v>
+        <v>8154.71258258538</v>
       </c>
       <c r="C10" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12)</f>
-        <v>1.91160165596738</v>
+        <v>1.42490460439143</v>
       </c>
       <c r="D10" s="50" t="n">
         <f aca="false">B10-$B$5</f>
@@ -5289,11 +5289,11 @@
       </c>
       <c r="B11" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Flächen und Mieten'!F23*(1-Annahmen!$B$48)</f>
-        <v>18098.8473035045</v>
+        <v>8758.22230350448</v>
       </c>
       <c r="C11" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-'Flächen und Mieten'!F23*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>2.0206103217238</v>
+        <v>1.49388405421695</v>
       </c>
       <c r="D11" s="50" t="n">
         <f aca="false">B11-$B$5</f>
@@ -5306,11 +5306,11 @@
       </c>
       <c r="B12" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48)</f>
-        <v>17513.8473035045</v>
+        <v>8173.22230350448</v>
       </c>
       <c r="C12" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.98762164414692</v>
+        <v>1.46089537664007</v>
       </c>
       <c r="D12" s="50" t="n">
         <f aca="false">B12-$B$5</f>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="D13" s="50" t="n">
         <f aca="false">B13-$B$5</f>
-        <v>-28658.675</v>
+        <v>-19318.05</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6517,7 +6517,7 @@
         <v>119</v>
       </c>
       <c r="B40" s="18" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>120</v>
@@ -6528,7 +6528,7 @@
         <v>121</v>
       </c>
       <c r="B41" s="18" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>122</v>
@@ -6612,7 +6612,7 @@
       </c>
       <c r="B49" s="21" t="n">
         <f aca="false">'Gastro Tagesteile'!F14</f>
-        <v>95635</v>
+        <v>65010</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>136</v>
@@ -7588,11 +7588,11 @@
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">Annahmen!$B$40</f>
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">B7*C7</f>
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H7" s="9"/>
     </row>
@@ -7605,11 +7605,11 @@
       </c>
       <c r="C8" s="36" t="n">
         <f aca="false">Annahmen!$B$41</f>
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="D8" s="28" t="n">
         <f aca="false">B8*C8</f>
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="H8" s="9"/>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="D17" s="33" t="n">
         <f aca="false">Annahmen!$B$49*12/D15</f>
-        <v>6040.1052631579</v>
+        <v>4105.89473684211</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>250</v>
@@ -7730,7 +7730,7 @@
       </c>
       <c r="D18" s="40" t="n">
         <f aca="false">'Flächen und Mieten'!F22/Annahmen!$B$49</f>
-        <v>0.0533277565744759</v>
+        <v>0.0784494693124135</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>252</v>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="D36" s="31" t="n">
         <f aca="false">(D5+D6+D7)/10</f>
-        <v>37.1</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="D38" s="45" t="n">
         <f aca="false">SUM(D35:D37)</f>
-        <v>54.6</v>
+        <v>56.6</v>
       </c>
       <c r="H38" s="9" t="s">
         <v>275</v>
@@ -37089,11 +37089,11 @@
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">'Gastro Betrieb'!C19</f>
-        <v>24068.675</v>
+        <v>14728.05</v>
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">B10*12</f>
-        <v>288824.1</v>
+        <v>176736.6</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>386</v>
@@ -37105,11 +37105,11 @@
       </c>
       <c r="B11" s="35" t="n">
         <f aca="false">B9+B10</f>
-        <v>36687.2044117647</v>
+        <v>27346.5794117647</v>
       </c>
       <c r="C11" s="35" t="n">
         <f aca="false">B11*12</f>
-        <v>440246.452941176</v>
+        <v>328158.952941176</v>
       </c>
       <c r="D11" s="9"/>
     </row>
@@ -37133,11 +37133,11 @@
       </c>
       <c r="B13" s="51" t="n">
         <f aca="false">B11+B12</f>
-        <v>18953.8473035045</v>
+        <v>9613.22230350448</v>
       </c>
       <c r="C13" s="52" t="n">
         <f aca="false">B13*12</f>
-        <v>227446.167642054</v>
+        <v>115358.667642054</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>389</v>
@@ -37149,7 +37149,7 @@
       </c>
       <c r="B15" s="53" t="n">
         <f aca="false">B11/-B12</f>
-        <v>2.06882454279769</v>
+        <v>1.54209827529084</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>40</v>
@@ -37185,7 +37185,7 @@
       </c>
       <c r="B18" s="55" t="n">
         <f aca="false">B11/('Tilgung Jahre'!B5/12)</f>
-        <v>2.69124680221824</v>
+        <v>2.00605076275363</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Revert "Gastro-Konzept: Frühstück und Bowls tagsüber, abends Bar mit Snacks; Umsatzmodell, Flächen, Personal angepasst"
This reverts commit 93b7f1f13931f73ad5737f3663b8d404f465e8a6.
</commit_message>
<xml_diff>
--- a/praesentation/Bankunterlagen_Baufeld3.xlsx
+++ b/praesentation/Bankunterlagen_Baufeld3.xlsx
@@ -397,13 +397,13 @@
     <t xml:space="preserve">Bar- und Theken-Zone (m²)</t>
   </si>
   <si>
-    <t xml:space="preserve">große Theke, Backbar, Service, Stehtische (Bar im Fokus)</t>
+    <t xml:space="preserve">Theke, Backbar, Service</t>
   </si>
   <si>
     <t xml:space="preserve">Küche mit Spülküche (m²)</t>
   </si>
   <si>
-    <t xml:space="preserve">kleine Bowl- und Snack-Küche, keine große Restaurantküche</t>
+    <t xml:space="preserve">Richtwert ca. 25–30 % der Gastraumfläche</t>
   </si>
   <si>
     <t xml:space="preserve">Lager, Kühlung, Anlieferung (m²)</t>
@@ -754,7 +754,7 @@
     <t xml:space="preserve">Bar und Theken-Zone</t>
   </si>
   <si>
-    <t xml:space="preserve">Küche (Bowls, Snacks) mit Spülküche</t>
+    <t xml:space="preserve">Küche mit Spülküche</t>
   </si>
   <si>
     <t xml:space="preserve">Lager, Kühlung, Anlieferung</t>
@@ -1303,10 +1303,10 @@
     <t xml:space="preserve">Bei sehr niedrigem Umsatz drücken Fixkosten stärker: die Rechnung ist dort zu günstig.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastro-Umsatz nach Tagesteilen: Frühstück, Mittag, Bar am Abend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tagsüber Frühstück und Bowls, abends Bar mit Snacks. Öffnungstage, Gäste und Bon sind Annahmen (keine Marktdaten für Werlte), Ruhetag Montag.</t>
+    <t xml:space="preserve">Gastro-Umsatz nach Tagesteilen: Frühstück, Mittag, Abend, Bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hauptfokus Abend mit Restaurant und Bar. Öffnungstage, Gäste und Bon sind Annahmen (keine Marktdaten für Werlte), Ruhetag Montag.</t>
   </si>
   <si>
     <t xml:space="preserve">Tagesteil</t>
@@ -1339,31 +1339,31 @@
     <t xml:space="preserve">Sa, So 09:00–14:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Mittag: Bowls, Salate, Suppe</t>
+    <t xml:space="preserve">Mittagstisch</t>
   </si>
   <si>
     <t xml:space="preserve">Di–Fr 11:30–14:30</t>
   </si>
   <si>
-    <t xml:space="preserve">Nachmittag: Kaffee, Kuchen, Snacks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Di–So 14:30–17:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bar mit Snacks Di–Do, So</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ab 17:00</t>
+    <t xml:space="preserve">Abendessen Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di–So 17:30–22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar Di–Do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ab 21:00</t>
   </si>
   <si>
     <t xml:space="preserve">Bar Fr, Sa (bis 01:00)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cocktails, Wein, Bier, Snacks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Events: Live-Musik, Feiern</t>
+    <t xml:space="preserve">Cocktails, Wein, Bier, Musik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feiern, Live-Abende, Séparée</t>
   </si>
   <si>
     <t xml:space="preserve">nach Absprache, 4 pro Monat</t>
@@ -1372,10 +1372,10 @@
     <t xml:space="preserve">Gastro-Umsatz pro Monat (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">davon Tag (Frühstück, Brunch, Mittag, Nachmittag)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">davon Abend (Bar mit Snacks, Events)</t>
+    <t xml:space="preserve">davon Tag (Frühstück, Brunch, Mittag)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">davon Abend (Restaurant, Bar, Feiern)</t>
   </si>
   <si>
     <t xml:space="preserve">Gäste pro Monat</t>
@@ -1384,10 +1384,10 @@
     <t xml:space="preserve">Umsatz je Platz und Jahr (190 Plätze)</t>
   </si>
   <si>
-    <t xml:space="preserve">Auslastung der Plätze an der Bar Fr, Sa (Gäste je Abend / Plätze)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Einordnung: Die Bar mit Snacks am Abend trägt den größten Teil des Umsatzes, Frühstück und Bowls füllen das Haus am Tag. Terrasse im Sommer, Catering und Weihnachtsfeiern sind nicht eingerechnet. Branchen-Median Österreich ca. 12.000 € je Platz und Jahr.</t>
+    <t xml:space="preserve">Auslastung der Plätze am Abend (Restaurantgäste je Tag / Plätze)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einordnung: Der Abend (Restaurant, Bar, Feiern) trägt den größten Teil des Umsatzes, Frühstück und Mittagstisch füllen das Haus am Tag. Terrasse im Sommer, Catering und Weihnachtsfeiern sind nicht eingerechnet. Branchen-Median Österreich ca. 12.000 € je Platz und Jahr.</t>
   </si>
   <si>
     <t xml:space="preserve">Ertragswert und Beleihung</t>
@@ -1756,7 +1756,7 @@
     <t xml:space="preserve">Projekt: Gastro-Konzept mit Gestaltung</t>
   </si>
   <si>
-    <t xml:space="preserve">Konzept (Frühstück, Bowls, Bar mit Snacks), Grundriss, Karte, Umsatzaufbau.</t>
+    <t xml:space="preserve">Konzept, Grundriss, Speisekarte, Umsatzaufbau.</t>
   </si>
   <si>
     <t xml:space="preserve">Projekt: Lageplan, Flurkarte, Grundbuchauszug</t>
@@ -2743,11 +2743,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="88830755"/>
-        <c:axId val="14380942"/>
+        <c:axId val="85622033"/>
+        <c:axId val="35587217"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="88830755"/>
+        <c:axId val="85622033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2813,7 +2813,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14380942"/>
+        <c:crossAx val="35587217"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2821,7 +2821,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14380942"/>
+        <c:axId val="35587217"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2897,7 +2897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88830755"/>
+        <c:crossAx val="85622033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">'Ertrag und Cashflow'!B10</f>
-        <v>14728.05</v>
+        <v>24068.675</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>37</v>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B25" s="13" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>9613.22230350448</v>
+        <v>18953.8473035045</v>
       </c>
       <c r="C25" s="9"/>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">'Ertrag und Cashflow'!B15</f>
-        <v>1.54209827529084</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>40</v>
@@ -3542,7 +3542,7 @@
       <c r="B5" s="7"/>
       <c r="C5" s="10" t="n">
         <f aca="false">Annahmen!$B$49</f>
-        <v>65010</v>
+        <v>95635</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="C6" s="33" t="n">
         <f aca="false">-$C$5*B6</f>
-        <v>-18202.8</v>
+        <v>-26777.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="C7" s="33" t="n">
         <f aca="false">-$C$5*B7</f>
-        <v>-19503</v>
+        <v>-28690.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="C8" s="33" t="n">
         <f aca="false">-$C$5*B8</f>
-        <v>-1950.3</v>
+        <v>-2869.05</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C9" s="33" t="n">
         <f aca="false">-$C$5*B9</f>
-        <v>-1300.2</v>
+        <v>-1912.7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">-$C$5*B10</f>
-        <v>-975.15</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C11" s="33" t="n">
         <f aca="false">-$C$5*B11</f>
-        <v>-975.15</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">-$C$5*B12</f>
-        <v>-975.15</v>
+        <v>-1434.525</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">-$C$5*B13</f>
-        <v>-650.1</v>
+        <v>-956.35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">-$C$5*B14</f>
-        <v>-650.1</v>
+        <v>-956.35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="C15" s="35" t="n">
         <f aca="false">SUM(C6:C14)</f>
-        <v>-45181.95</v>
+        <v>-66466.325</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="C16" s="35" t="n">
         <f aca="false">C5+C15</f>
-        <v>19828.05</v>
+        <v>29168.675</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>414</v>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C19" s="46" t="n">
         <f aca="false">C16+C17+C18</f>
-        <v>14728.05</v>
+        <v>24068.675</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3732,68 +3732,68 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="C24" s="33" t="n">
         <f aca="false">A24*$B$16</f>
-        <v>12200</v>
+        <v>15250</v>
       </c>
       <c r="D24" s="50" t="n">
         <f aca="false">C24-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>7100</v>
+        <v>10150</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="n">
-        <v>50000</v>
+        <v>65000</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">A25*$B$16</f>
-        <v>15250</v>
+        <v>19825</v>
       </c>
       <c r="D25" s="50" t="n">
         <f aca="false">C25-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>10150</v>
+        <v>14725</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="n">
-        <f aca="false">Annahmen!$B$49</f>
-        <v>65010</v>
+        <v>80000</v>
       </c>
       <c r="C26" s="33" t="n">
         <f aca="false">A26*$B$16</f>
-        <v>19828.05</v>
+        <v>24400</v>
       </c>
       <c r="D26" s="50" t="n">
         <f aca="false">C26-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>14728.05</v>
+        <v>19300</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="n">
-        <v>80000</v>
+        <f aca="false">Annahmen!$B$49</f>
+        <v>95635</v>
       </c>
       <c r="C27" s="33" t="n">
         <f aca="false">A27*$B$16</f>
-        <v>24400</v>
+        <v>29168.675</v>
       </c>
       <c r="D27" s="50" t="n">
         <f aca="false">C27-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>19300</v>
+        <v>24068.675</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="n">
-        <v>95000</v>
+        <v>110000</v>
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">A28*$B$16</f>
-        <v>28975</v>
+        <v>33550</v>
       </c>
       <c r="D28" s="50" t="n">
         <f aca="false">C28-'Flächen und Mieten'!$F$22-Annahmen!$B$51</f>
-        <v>23875</v>
+        <v>28450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3872,18 +3872,18 @@
         <v>17</v>
       </c>
       <c r="D5" s="57" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E5" s="19" t="n">
         <v>11</v>
       </c>
       <c r="F5" s="33" t="n">
         <f aca="false">C5*D5*E5</f>
-        <v>5610</v>
+        <v>4675</v>
       </c>
       <c r="G5" s="40" t="n">
         <f aca="false">F5/$F$14</f>
-        <v>0.0862944162436548</v>
+        <v>0.0488837768599362</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="G6" s="40" t="n">
         <f aca="false">F6/$F$14</f>
-        <v>0.116289801568989</v>
+        <v>0.0790505568045172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3922,18 +3922,18 @@
         <v>17</v>
       </c>
       <c r="D7" s="57" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="33" t="n">
         <f aca="false">C7*D7*E7</f>
-        <v>8840</v>
+        <v>11900</v>
       </c>
       <c r="G7" s="40" t="n">
         <f aca="false">F7/$F$14</f>
-        <v>0.135979080141517</v>
+        <v>0.12443143200711</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,18 +3947,18 @@
         <v>26</v>
       </c>
       <c r="D8" s="57" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="F8" s="33" t="n">
         <f aca="false">C8*D8*E8</f>
-        <v>3640</v>
+        <v>45760</v>
       </c>
       <c r="G8" s="40" t="n">
         <f aca="false">F8/$F$14</f>
-        <v>0.0559913859406245</v>
+        <v>0.478485909970199</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3969,21 +3969,21 @@
         <v>439</v>
       </c>
       <c r="C9" s="57" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D9" s="57" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">C9*D9*E9</f>
-        <v>11900</v>
+        <v>4680</v>
       </c>
       <c r="G9" s="40" t="n">
         <f aca="false">F9/$F$14</f>
-        <v>0.183048761728965</v>
+        <v>0.0489360589742249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3997,18 +3997,18 @@
         <v>9</v>
       </c>
       <c r="D10" s="57" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F10" s="33" t="n">
         <f aca="false">C10*D10*E10</f>
-        <v>21060</v>
+        <v>13860</v>
       </c>
       <c r="G10" s="40" t="n">
         <f aca="false">F10/$F$14</f>
-        <v>0.323950161513613</v>
+        <v>0.144926020808281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4025,15 +4025,15 @@
         <v>40</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F11" s="33" t="n">
         <f aca="false">C11*D11*E11</f>
-        <v>6400</v>
+        <v>7200</v>
       </c>
       <c r="G11" s="40" t="n">
         <f aca="false">F11/$F$14</f>
-        <v>0.0984463928626365</v>
+        <v>0.0752862445757307</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F14" s="46" t="n">
         <f aca="false">SUM(F5:F11)</f>
-        <v>65010</v>
+        <v>95635</v>
       </c>
       <c r="G14" s="42" t="n">
         <f aca="false">SUM(G5:G11)</f>
@@ -4054,12 +4054,12 @@
         <v>445</v>
       </c>
       <c r="F15" s="33" t="n">
-        <f aca="false">SUM(F5:F8)</f>
-        <v>25650</v>
+        <f aca="false">SUM(F5:F7)</f>
+        <v>24135</v>
       </c>
       <c r="G15" s="40" t="n">
         <f aca="false">F15/F14</f>
-        <v>0.394554683894785</v>
+        <v>0.252365765671564</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,12 +4067,12 @@
         <v>446</v>
       </c>
       <c r="F16" s="35" t="n">
-        <f aca="false">SUM(F9:F11)</f>
-        <v>39360</v>
+        <f aca="false">SUM(F8:F11)</f>
+        <v>71500</v>
       </c>
       <c r="G16" s="42" t="n">
         <f aca="false">F16/F14</f>
-        <v>0.605445316105215</v>
+        <v>0.747634234328436</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="F17" s="28" t="n">
         <f aca="false">SUMPRODUCT(C5:C11,D5:D11)</f>
-        <v>3815</v>
+        <v>4295</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="F18" s="33" t="n">
         <f aca="false">F14*12/(Annahmen!$B$36+Annahmen!$B$37)</f>
-        <v>4105.89473684211</v>
+        <v>6040.1052631579</v>
       </c>
       <c r="G18" s="9"/>
     </row>
@@ -4099,8 +4099,8 @@
         <v>449</v>
       </c>
       <c r="F19" s="40" t="n">
-        <f aca="false">D10/(Annahmen!$B$36+Annahmen!$B$37)</f>
-        <v>0.473684210526316</v>
+        <f aca="false">D8/(Annahmen!$B$36+Annahmen!$B$37)</f>
+        <v>0.289473684210526</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4866,43 +4866,43 @@
       </c>
       <c r="B9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(1-1))-B7-Annahmen!$B$51*12</f>
-        <v>176736.6</v>
+        <v>288824.1</v>
       </c>
       <c r="C9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(2-1))-C7-Annahmen!$B$51*12</f>
-        <v>179387.649</v>
+        <v>293156.4615</v>
       </c>
       <c r="D9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(3-1))-D7-Annahmen!$B$51*12</f>
-        <v>182078.463735</v>
+        <v>297553.8084225</v>
       </c>
       <c r="E9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(4-1))-E7-Annahmen!$B$51*12</f>
-        <v>184809.640691025</v>
+        <v>302017.115548837</v>
       </c>
       <c r="F9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(5-1))-F7-Annahmen!$B$51*12</f>
-        <v>187581.78530139</v>
+        <v>306547.37228207</v>
       </c>
       <c r="G9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(6-1))-G7-Annahmen!$B$51*12</f>
-        <v>190395.512080911</v>
+        <v>311145.582866301</v>
       </c>
       <c r="H9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(7-1))-H7-Annahmen!$B$51*12</f>
-        <v>193251.444762125</v>
+        <v>315812.766609295</v>
       </c>
       <c r="I9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(8-1))-I7-Annahmen!$B$51*12</f>
-        <v>196150.216433557</v>
+        <v>320549.958108435</v>
       </c>
       <c r="J9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(9-1))-J7-Annahmen!$B$51*12</f>
-        <v>199092.46968006</v>
+        <v>325358.207480061</v>
       </c>
       <c r="K9" s="33" t="n">
         <f aca="false">('Gastro Betrieb'!$C$16*12*(1+Annahmen!$B$79)^(10-1))-K7-Annahmen!$B$51*12</f>
-        <v>202078.856725261</v>
+        <v>330238.580592262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4911,43 +4911,43 @@
       </c>
       <c r="B10" s="35" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>328158.952941176</v>
+        <v>440246.452941176</v>
       </c>
       <c r="C10" s="35" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>333167.737235294</v>
+        <v>446936.549735294</v>
       </c>
       <c r="D10" s="35" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>338253.381293823</v>
+        <v>453728.725981323</v>
       </c>
       <c r="E10" s="35" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>343417.072573231</v>
+        <v>460624.547431043</v>
       </c>
       <c r="F10" s="35" t="n">
         <f aca="false">SUM(F5:F9)</f>
-        <v>348660.017033029</v>
+        <v>467625.604013709</v>
       </c>
       <c r="G10" s="35" t="n">
         <f aca="false">SUM(G5:G9)</f>
-        <v>353983.439427149</v>
+        <v>474733.510212538</v>
       </c>
       <c r="H10" s="35" t="n">
         <f aca="false">SUM(H5:H9)</f>
-        <v>359388.583599952</v>
+        <v>481949.905447123</v>
       </c>
       <c r="I10" s="35" t="n">
         <f aca="false">SUM(I5:I9)</f>
-        <v>364876.712786976</v>
+        <v>489276.454461854</v>
       </c>
       <c r="J10" s="35" t="n">
         <f aca="false">SUM(J5:J9)</f>
-        <v>370449.109920465</v>
+        <v>496714.847720467</v>
       </c>
       <c r="K10" s="35" t="n">
         <f aca="false">SUM(K5:K9)</f>
-        <v>376107.077939791</v>
+        <v>504266.801806792</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5001,43 +5001,43 @@
       </c>
       <c r="B12" s="52" t="n">
         <f aca="false">B10+B11</f>
-        <v>115358.667642054</v>
+        <v>227446.167642054</v>
       </c>
       <c r="C12" s="52" t="n">
         <f aca="false">C10+C11</f>
-        <v>120367.451936171</v>
+        <v>234136.264436171</v>
       </c>
       <c r="D12" s="52" t="n">
         <f aca="false">D10+D11</f>
-        <v>125453.095994701</v>
+        <v>240928.440682201</v>
       </c>
       <c r="E12" s="52" t="n">
         <f aca="false">E10+E11</f>
-        <v>130616.787274108</v>
+        <v>247824.26213192</v>
       </c>
       <c r="F12" s="52" t="n">
         <f aca="false">F10+F11</f>
-        <v>135859.731733907</v>
+        <v>254825.318714586</v>
       </c>
       <c r="G12" s="52" t="n">
         <f aca="false">G10+G11</f>
-        <v>141183.154128026</v>
+        <v>261933.224913416</v>
       </c>
       <c r="H12" s="52" t="n">
         <f aca="false">H10+H11</f>
-        <v>146588.298300829</v>
+        <v>269149.620148</v>
       </c>
       <c r="I12" s="52" t="n">
         <f aca="false">I10+I11</f>
-        <v>152076.427487853</v>
+        <v>276476.169162731</v>
       </c>
       <c r="J12" s="52" t="n">
         <f aca="false">J10+J11</f>
-        <v>157648.824621343</v>
+        <v>283914.562421344</v>
       </c>
       <c r="K12" s="52" t="n">
         <f aca="false">K10+K11</f>
-        <v>163306.792640668</v>
+        <v>291466.516507669</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5046,43 +5046,43 @@
       </c>
       <c r="B13" s="54" t="n">
         <f aca="false">B10/-B11</f>
-        <v>1.54209827529084</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="C13" s="54" t="n">
         <f aca="false">C10/-C11</f>
-        <v>1.56563576391346</v>
+        <v>2.10026292543291</v>
       </c>
       <c r="D13" s="54" t="n">
         <f aca="false">D10/-D11</f>
-        <v>1.58953443515528</v>
+        <v>2.13218100409753</v>
       </c>
       <c r="E13" s="54" t="n">
         <f aca="false">E10/-E11</f>
-        <v>1.61379986916139</v>
+        <v>2.16458613663777</v>
       </c>
       <c r="F13" s="54" t="n">
         <f aca="false">F10/-F11</f>
-        <v>1.63843773302717</v>
+        <v>2.19748579451569</v>
       </c>
       <c r="G13" s="54" t="n">
         <f aca="false">G10/-G11</f>
-        <v>1.6634537821675</v>
+        <v>2.23088756457835</v>
       </c>
       <c r="H13" s="54" t="n">
         <f aca="false">H10/-H11</f>
-        <v>1.68885386170783</v>
+        <v>2.26479915085485</v>
       </c>
       <c r="I13" s="54" t="n">
         <f aca="false">I10/-I11</f>
-        <v>1.71464390789743</v>
+        <v>2.29922837638165</v>
       </c>
       <c r="J13" s="54" t="n">
         <f aca="false">J10/-J11</f>
-        <v>1.74082994954515</v>
+        <v>2.33418318505663</v>
       </c>
       <c r="K13" s="54" t="n">
         <f aca="false">K10/-K11</f>
-        <v>1.76741810947817</v>
+        <v>2.36967164352233</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5190,11 +5190,11 @@
       </c>
       <c r="B5" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13</f>
-        <v>9613.22230350448</v>
+        <v>18953.8473035045</v>
       </c>
       <c r="C5" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/Tilgungsplan!N3</f>
-        <v>1.54209827529084</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="D5" s="50"/>
     </row>
@@ -5204,11 +5204,11 @@
       </c>
       <c r="B6" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Tilgung Jahre'!E14*0.01/12</f>
-        <v>6055.57203384148</v>
+        <v>15396.1970338415</v>
       </c>
       <c r="C6" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+'Tilgung Jahre'!E14*0.01/12)</f>
-        <v>1.28441923514246</v>
+        <v>1.72313144984421</v>
       </c>
       <c r="D6" s="50" t="n">
         <f aca="false">B6-$B$5</f>
@@ -5221,15 +5221,15 @@
       </c>
       <c r="B7" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48)</f>
-        <v>8954.36936232801</v>
+        <v>18294.994362328</v>
       </c>
       <c r="C7" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.1*'Ertrag und Cashflow'!B5*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.50494496375743</v>
+        <v>2.03167123126428</v>
       </c>
       <c r="D7" s="50" t="n">
         <f aca="false">B7-$B$5</f>
-        <v>-658.85294117647</v>
+        <v>-658.852941176472</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,15 +5238,15 @@
       </c>
       <c r="B8" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.2*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>5647.61230350448</v>
+        <v>13120.1123035045</v>
       </c>
       <c r="C8" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.2*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.31847395104189</v>
+        <v>1.73985496504737</v>
       </c>
       <c r="D8" s="50" t="n">
         <f aca="false">B8-$B$5</f>
-        <v>-3965.61</v>
+        <v>-5833.735</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5255,15 +5255,15 @@
       </c>
       <c r="B9" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.4*Annahmen!$B$49*Annahmen!$B$50</f>
-        <v>1682.00230350448</v>
+        <v>7286.37730350447</v>
       </c>
       <c r="C9" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-0.4*Annahmen!$B$49*Annahmen!$B$50)/Tilgungsplan!N3</f>
-        <v>1.09484962679294</v>
+        <v>1.41088538729705</v>
       </c>
       <c r="D9" s="50" t="n">
         <f aca="false">B9-$B$5</f>
-        <v>-7931.22</v>
+        <v>-11667.47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5272,11 +5272,11 @@
       </c>
       <c r="B10" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12</f>
-        <v>8154.71258258538</v>
+        <v>17495.3375825854</v>
       </c>
       <c r="C10" s="55" t="n">
         <f aca="false">'Ertrag und Cashflow'!B11/(Tilgungsplan!N3+0.1*'Kosten und Finanzierung'!B12*(1+Annahmen!$B$17)*('Kosten und Finanzierung'!B31+Annahmen!$B$58)/12)</f>
-        <v>1.42490460439143</v>
+        <v>1.91160165596738</v>
       </c>
       <c r="D10" s="50" t="n">
         <f aca="false">B10-$B$5</f>
@@ -5289,11 +5289,11 @@
       </c>
       <c r="B11" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Flächen und Mieten'!F23*(1-Annahmen!$B$48)</f>
-        <v>8758.22230350448</v>
+        <v>18098.8473035045</v>
       </c>
       <c r="C11" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-'Flächen und Mieten'!F23*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.49388405421695</v>
+        <v>2.0206103217238</v>
       </c>
       <c r="D11" s="50" t="n">
         <f aca="false">B11-$B$5</f>
@@ -5306,11 +5306,11 @@
       </c>
       <c r="B12" s="50" t="n">
         <f aca="false">'Ertrag und Cashflow'!B13-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48)</f>
-        <v>8173.22230350448</v>
+        <v>17513.8473035045</v>
       </c>
       <c r="C12" s="55" t="n">
         <f aca="false">('Ertrag und Cashflow'!B11-'Ertrag und Cashflow'!B6*(1-Annahmen!$B$48))/Tilgungsplan!N3</f>
-        <v>1.46089537664007</v>
+        <v>1.98762164414692</v>
       </c>
       <c r="D12" s="50" t="n">
         <f aca="false">B12-$B$5</f>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="D13" s="50" t="n">
         <f aca="false">B13-$B$5</f>
-        <v>-19318.05</v>
+        <v>-28658.675</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6517,7 +6517,7 @@
         <v>119</v>
       </c>
       <c r="B40" s="18" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>120</v>
@@ -6528,7 +6528,7 @@
         <v>121</v>
       </c>
       <c r="B41" s="18" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>122</v>
@@ -6612,7 +6612,7 @@
       </c>
       <c r="B49" s="21" t="n">
         <f aca="false">'Gastro Tagesteile'!F14</f>
-        <v>65010</v>
+        <v>95635</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>136</v>
@@ -7588,11 +7588,11 @@
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">Annahmen!$B$40</f>
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">B7*C7</f>
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H7" s="9"/>
     </row>
@@ -7605,11 +7605,11 @@
       </c>
       <c r="C8" s="36" t="n">
         <f aca="false">Annahmen!$B$41</f>
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="D8" s="28" t="n">
         <f aca="false">B8*C8</f>
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H8" s="9"/>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="D17" s="33" t="n">
         <f aca="false">Annahmen!$B$49*12/D15</f>
-        <v>4105.89473684211</v>
+        <v>6040.1052631579</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>250</v>
@@ -7730,7 +7730,7 @@
       </c>
       <c r="D18" s="40" t="n">
         <f aca="false">'Flächen und Mieten'!F22/Annahmen!$B$49</f>
-        <v>0.0784494693124135</v>
+        <v>0.0533277565744759</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>252</v>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="D36" s="31" t="n">
         <f aca="false">(D5+D6+D7)/10</f>
-        <v>39.1</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="D38" s="45" t="n">
         <f aca="false">SUM(D35:D37)</f>
-        <v>56.6</v>
+        <v>54.6</v>
       </c>
       <c r="H38" s="9" t="s">
         <v>275</v>
@@ -37089,11 +37089,11 @@
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">'Gastro Betrieb'!C19</f>
-        <v>14728.05</v>
+        <v>24068.675</v>
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">B10*12</f>
-        <v>176736.6</v>
+        <v>288824.1</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>386</v>
@@ -37105,11 +37105,11 @@
       </c>
       <c r="B11" s="35" t="n">
         <f aca="false">B9+B10</f>
-        <v>27346.5794117647</v>
+        <v>36687.2044117647</v>
       </c>
       <c r="C11" s="35" t="n">
         <f aca="false">B11*12</f>
-        <v>328158.952941176</v>
+        <v>440246.452941176</v>
       </c>
       <c r="D11" s="9"/>
     </row>
@@ -37133,11 +37133,11 @@
       </c>
       <c r="B13" s="51" t="n">
         <f aca="false">B11+B12</f>
-        <v>9613.22230350448</v>
+        <v>18953.8473035045</v>
       </c>
       <c r="C13" s="52" t="n">
         <f aca="false">B13*12</f>
-        <v>115358.667642054</v>
+        <v>227446.167642054</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>389</v>
@@ -37149,7 +37149,7 @@
       </c>
       <c r="B15" s="53" t="n">
         <f aca="false">B11/-B12</f>
-        <v>1.54209827529084</v>
+        <v>2.06882454279769</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>40</v>
@@ -37185,7 +37185,7 @@
       </c>
       <c r="B18" s="55" t="n">
         <f aca="false">B11/('Tilgung Jahre'!B5/12)</f>
-        <v>2.00605076275363</v>
+        <v>2.69124680221824</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>